<commit_message>
Ship attendance day snapshots on Process, payroll reports, and Pulse 0.1.58.
Persist daily OT/late/undertime metrics to trn_payroll_attendance_days for Attendance View and reports, and bump the paired desktop installers.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/templates/employee_upload_template.xlsx
+++ b/resources/templates/employee_upload_template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="292">
   <si>
     <t>employee_number</t>
   </si>
@@ -107,6 +107,51 @@
     <t>campus2_program</t>
   </si>
   <si>
+    <t>campus3_code</t>
+  </si>
+  <si>
+    <t>campus3_biometric_id</t>
+  </si>
+  <si>
+    <t>campus3_college</t>
+  </si>
+  <si>
+    <t>campus3_department</t>
+  </si>
+  <si>
+    <t>campus3_program</t>
+  </si>
+  <si>
+    <t>campus4_code</t>
+  </si>
+  <si>
+    <t>campus4_biometric_id</t>
+  </si>
+  <si>
+    <t>campus4_college</t>
+  </si>
+  <si>
+    <t>campus4_department</t>
+  </si>
+  <si>
+    <t>campus4_program</t>
+  </si>
+  <si>
+    <t>campus5_code</t>
+  </si>
+  <si>
+    <t>campus5_biometric_id</t>
+  </si>
+  <si>
+    <t>campus5_college</t>
+  </si>
+  <si>
+    <t>campus5_department</t>
+  </si>
+  <si>
+    <t>campus5_program</t>
+  </si>
+  <si>
     <t>is_hybrid</t>
   </si>
   <si>
@@ -176,6 +221,9 @@
     <t>salary_use_basic_income_as_hourly_rate</t>
   </si>
   <si>
+    <t>salary_is_above_minimum_wage_earner</t>
+  </si>
+  <si>
     <t>salary_basic_taxable</t>
   </si>
   <si>
@@ -215,6 +263,9 @@
     <t>salary2_use_basic_income_as_hourly_rate</t>
   </si>
   <si>
+    <t>salary2_is_above_minimum_wage_earner</t>
+  </si>
+  <si>
     <t>salary2_basic_taxable</t>
   </si>
   <si>
@@ -371,24 +422,6 @@
     <t>gi_organization_memberships</t>
   </si>
   <si>
-    <t>json_family_members</t>
-  </si>
-  <si>
-    <t>json_employment_history</t>
-  </si>
-  <si>
-    <t>json_exams</t>
-  </si>
-  <si>
-    <t>json_seminars</t>
-  </si>
-  <si>
-    <t>json_awards</t>
-  </si>
-  <si>
-    <t>json_references</t>
-  </si>
-  <si>
     <t>Employee Number</t>
   </si>
   <si>
@@ -479,6 +512,51 @@
     <t>Program 2</t>
   </si>
   <si>
+    <t>Campus Code 3</t>
+  </si>
+  <si>
+    <t>Biometric ID 3</t>
+  </si>
+  <si>
+    <t>Department / College 3</t>
+  </si>
+  <si>
+    <t>Employee Department 3</t>
+  </si>
+  <si>
+    <t>Program 3</t>
+  </si>
+  <si>
+    <t>Campus Code 4</t>
+  </si>
+  <si>
+    <t>Biometric ID 4</t>
+  </si>
+  <si>
+    <t>Department / College 4</t>
+  </si>
+  <si>
+    <t>Employee Department 4</t>
+  </si>
+  <si>
+    <t>Program 4</t>
+  </si>
+  <si>
+    <t>Campus Code 5</t>
+  </si>
+  <si>
+    <t>Biometric ID 5</t>
+  </si>
+  <si>
+    <t>Department / College 5</t>
+  </si>
+  <si>
+    <t>Employee Department 5</t>
+  </si>
+  <si>
+    <t>Program 5</t>
+  </si>
+  <si>
     <t>Hybrid (yes/no)</t>
   </si>
   <si>
@@ -548,6 +626,9 @@
     <t>Use Basic Income as Hourly Rate (yes/no)</t>
   </si>
   <si>
+    <t>Is Above Minimum Wage Earner (yes/no)</t>
+  </si>
+  <si>
     <t>Basic Income Taxable</t>
   </si>
   <si>
@@ -587,6 +668,9 @@
     <t>Use Basic Income as Hourly Rate 2 (yes/no)</t>
   </si>
   <si>
+    <t>Is Above Minimum Wage Earner 2 (yes/no)</t>
+  </si>
+  <si>
     <t>Basic Income Taxable 2</t>
   </si>
   <si>
@@ -741,24 +825,6 @@
   </si>
   <si>
     <t>Organization Memberships</t>
-  </si>
-  <si>
-    <t>Family Members JSON</t>
-  </si>
-  <si>
-    <t>Employment History JSON</t>
-  </si>
-  <si>
-    <t>Exams JSON</t>
-  </si>
-  <si>
-    <t>Seminars JSON</t>
-  </si>
-  <si>
-    <t>Awards JSON</t>
-  </si>
-  <si>
-    <t>References JSON</t>
   </si>
   <si>
     <t>2026-00099</t>
@@ -1165,10 +1231,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:DT150"/>
+  <dimension ref="A1:EE150"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:124">
+    <row r="1" spans="1:135">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1541,453 +1607,519 @@
       <c r="DT1" t="s">
         <v>123</v>
       </c>
+      <c r="DU1" t="s">
+        <v>124</v>
+      </c>
+      <c r="DV1" t="s">
+        <v>125</v>
+      </c>
+      <c r="DW1" t="s">
+        <v>126</v>
+      </c>
+      <c r="DX1" t="s">
+        <v>127</v>
+      </c>
+      <c r="DY1" t="s">
+        <v>128</v>
+      </c>
+      <c r="DZ1" t="s">
+        <v>129</v>
+      </c>
+      <c r="EA1" t="s">
+        <v>130</v>
+      </c>
+      <c r="EB1" t="s">
+        <v>131</v>
+      </c>
+      <c r="EC1" t="s">
+        <v>132</v>
+      </c>
+      <c r="ED1" t="s">
+        <v>133</v>
+      </c>
+      <c r="EE1" t="s">
+        <v>134</v>
+      </c>
     </row>
-    <row r="2" spans="1:124">
+    <row r="2" spans="1:135">
       <c r="A2" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="C2" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="D2" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="E2" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="F2" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="G2" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="H2" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="I2" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="J2" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="K2" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="L2" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="M2" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="N2" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="O2" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="P2" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="Q2" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="R2" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="S2" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="T2" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="U2" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="V2" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="W2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="X2" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="Y2" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="Z2" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="AA2" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="AB2" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="AC2" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="AD2" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="AE2" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="AF2" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="AG2" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="AH2" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="AI2" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="AJ2" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="AK2" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="AL2" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="AM2" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="AN2" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="AO2" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="AP2" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="AQ2" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="AR2" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="AS2" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="AT2" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="AU2" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="AV2" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="AW2" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="AX2" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="AY2" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="AZ2" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="BA2" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="BB2" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="BC2" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="BD2" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="BE2" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="BF2" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="BG2" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="BH2" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="BI2" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="BJ2" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="BK2" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="BL2" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="BM2" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="BN2" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="BO2" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="BP2" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="BQ2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="BR2" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="BS2" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="BT2" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="BU2" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="BV2" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="BW2" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="BX2" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="BY2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="BZ2" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="CA2" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="CB2" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="CC2" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="CD2" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="CE2" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="CF2" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="CG2" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="CH2" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="CI2" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="CJ2" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="CK2" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="CL2" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="CM2" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="CN2" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="CO2" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="CP2" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="CQ2" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="CR2" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="CS2" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="CT2" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="CU2" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="CV2" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="CW2" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="CX2" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="CY2" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="CZ2" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="DA2" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="DB2" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="DC2" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="DD2" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="DE2" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="DF2" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="DG2" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="DH2" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="DI2" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="DJ2" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
       <c r="DK2" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="DL2" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
       <c r="DM2" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="DN2" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="DO2" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="DP2" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
       <c r="DQ2" t="s">
-        <v>244</v>
+        <v>255</v>
       </c>
       <c r="DR2" t="s">
-        <v>245</v>
+        <v>256</v>
       </c>
       <c r="DS2" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="DT2" t="s">
-        <v>247</v>
+        <v>258</v>
+      </c>
+      <c r="DU2" t="s">
+        <v>259</v>
+      </c>
+      <c r="DV2" t="s">
+        <v>260</v>
+      </c>
+      <c r="DW2" t="s">
+        <v>261</v>
+      </c>
+      <c r="DX2" t="s">
+        <v>262</v>
+      </c>
+      <c r="DY2" t="s">
+        <v>263</v>
+      </c>
+      <c r="DZ2" t="s">
+        <v>264</v>
+      </c>
+      <c r="EA2" t="s">
+        <v>265</v>
+      </c>
+      <c r="EB2" t="s">
+        <v>266</v>
+      </c>
+      <c r="EC2" t="s">
+        <v>267</v>
+      </c>
+      <c r="ED2" t="s">
+        <v>268</v>
+      </c>
+      <c r="EE2" t="s">
+        <v>269</v>
       </c>
     </row>
-    <row r="3" spans="1:124">
+    <row r="3" spans="1:135">
       <c r="A3" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
       <c r="B3" t="s">
-        <v>249</v>
+        <v>271</v>
       </c>
       <c r="C3" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="D3" t="s">
-        <v>251</v>
+        <v>273</v>
       </c>
       <c r="U3" t="s">
-        <v>252</v>
+        <v>274</v>
       </c>
       <c r="V3" t="s">
-        <v>253</v>
+        <v>275</v>
       </c>
       <c r="W3" t="s">
-        <v>254</v>
+        <v>276</v>
       </c>
       <c r="X3" t="s">
-        <v>254</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>255</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>256</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>257</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>258</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>259</v>
+        <v>276</v>
+      </c>
+      <c r="AT3" t="s">
+        <v>277</v>
       </c>
       <c r="AU3" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="AV3" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
       <c r="AW3" t="s">
-        <v>262</v>
-      </c>
-      <c r="AZ3" t="s">
-        <v>263</v>
-      </c>
-      <c r="BB3" t="s">
-        <v>264</v>
-      </c>
-      <c r="BS3" t="s">
-        <v>265</v>
-      </c>
-      <c r="BT3" t="s">
-        <v>266</v>
-      </c>
-      <c r="CC3" t="s">
-        <v>267</v>
+        <v>280</v>
+      </c>
+      <c r="BH3" t="s">
+        <v>281</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>282</v>
+      </c>
+      <c r="BK3" t="s">
+        <v>283</v>
+      </c>
+      <c r="BL3" t="s">
+        <v>284</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>285</v>
+      </c>
+      <c r="BR3" t="s">
+        <v>286</v>
       </c>
       <c r="CJ3" t="s">
-        <v>268</v>
-      </c>
-      <c r="CL3" t="s">
-        <v>269</v>
+        <v>287</v>
+      </c>
+      <c r="CK3" t="s">
+        <v>288</v>
+      </c>
+      <c r="CT3" t="s">
+        <v>289</v>
+      </c>
+      <c r="DA3" t="s">
+        <v>290</v>
+      </c>
+      <c r="DC3" t="s">
+        <v>291</v>
       </c>
     </row>
-    <row r="4" spans="1:124">
+    <row r="4" spans="1:135">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -2112,8 +2244,19 @@
       <c r="DR4" s="1"/>
       <c r="DS4" s="1"/>
       <c r="DT4" s="1"/>
+      <c r="DU4" s="1"/>
+      <c r="DV4" s="1"/>
+      <c r="DW4" s="1"/>
+      <c r="DX4" s="1"/>
+      <c r="DY4" s="1"/>
+      <c r="DZ4" s="1"/>
+      <c r="EA4" s="1"/>
+      <c r="EB4" s="1"/>
+      <c r="EC4" s="1"/>
+      <c r="ED4" s="1"/>
+      <c r="EE4" s="1"/>
     </row>
-    <row r="5" spans="1:124">
+    <row r="5" spans="1:135">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -2238,8 +2381,19 @@
       <c r="DR5" s="1"/>
       <c r="DS5" s="1"/>
       <c r="DT5" s="1"/>
+      <c r="DU5" s="1"/>
+      <c r="DV5" s="1"/>
+      <c r="DW5" s="1"/>
+      <c r="DX5" s="1"/>
+      <c r="DY5" s="1"/>
+      <c r="DZ5" s="1"/>
+      <c r="EA5" s="1"/>
+      <c r="EB5" s="1"/>
+      <c r="EC5" s="1"/>
+      <c r="ED5" s="1"/>
+      <c r="EE5" s="1"/>
     </row>
-    <row r="6" spans="1:124">
+    <row r="6" spans="1:135">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -2364,8 +2518,19 @@
       <c r="DR6" s="1"/>
       <c r="DS6" s="1"/>
       <c r="DT6" s="1"/>
+      <c r="DU6" s="1"/>
+      <c r="DV6" s="1"/>
+      <c r="DW6" s="1"/>
+      <c r="DX6" s="1"/>
+      <c r="DY6" s="1"/>
+      <c r="DZ6" s="1"/>
+      <c r="EA6" s="1"/>
+      <c r="EB6" s="1"/>
+      <c r="EC6" s="1"/>
+      <c r="ED6" s="1"/>
+      <c r="EE6" s="1"/>
     </row>
-    <row r="7" spans="1:124">
+    <row r="7" spans="1:135">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -2490,8 +2655,19 @@
       <c r="DR7" s="1"/>
       <c r="DS7" s="1"/>
       <c r="DT7" s="1"/>
+      <c r="DU7" s="1"/>
+      <c r="DV7" s="1"/>
+      <c r="DW7" s="1"/>
+      <c r="DX7" s="1"/>
+      <c r="DY7" s="1"/>
+      <c r="DZ7" s="1"/>
+      <c r="EA7" s="1"/>
+      <c r="EB7" s="1"/>
+      <c r="EC7" s="1"/>
+      <c r="ED7" s="1"/>
+      <c r="EE7" s="1"/>
     </row>
-    <row r="8" spans="1:124">
+    <row r="8" spans="1:135">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -2616,8 +2792,19 @@
       <c r="DR8" s="1"/>
       <c r="DS8" s="1"/>
       <c r="DT8" s="1"/>
+      <c r="DU8" s="1"/>
+      <c r="DV8" s="1"/>
+      <c r="DW8" s="1"/>
+      <c r="DX8" s="1"/>
+      <c r="DY8" s="1"/>
+      <c r="DZ8" s="1"/>
+      <c r="EA8" s="1"/>
+      <c r="EB8" s="1"/>
+      <c r="EC8" s="1"/>
+      <c r="ED8" s="1"/>
+      <c r="EE8" s="1"/>
     </row>
-    <row r="9" spans="1:124">
+    <row r="9" spans="1:135">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -2742,8 +2929,19 @@
       <c r="DR9" s="1"/>
       <c r="DS9" s="1"/>
       <c r="DT9" s="1"/>
+      <c r="DU9" s="1"/>
+      <c r="DV9" s="1"/>
+      <c r="DW9" s="1"/>
+      <c r="DX9" s="1"/>
+      <c r="DY9" s="1"/>
+      <c r="DZ9" s="1"/>
+      <c r="EA9" s="1"/>
+      <c r="EB9" s="1"/>
+      <c r="EC9" s="1"/>
+      <c r="ED9" s="1"/>
+      <c r="EE9" s="1"/>
     </row>
-    <row r="10" spans="1:124">
+    <row r="10" spans="1:135">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -2868,8 +3066,19 @@
       <c r="DR10" s="1"/>
       <c r="DS10" s="1"/>
       <c r="DT10" s="1"/>
+      <c r="DU10" s="1"/>
+      <c r="DV10" s="1"/>
+      <c r="DW10" s="1"/>
+      <c r="DX10" s="1"/>
+      <c r="DY10" s="1"/>
+      <c r="DZ10" s="1"/>
+      <c r="EA10" s="1"/>
+      <c r="EB10" s="1"/>
+      <c r="EC10" s="1"/>
+      <c r="ED10" s="1"/>
+      <c r="EE10" s="1"/>
     </row>
-    <row r="11" spans="1:124">
+    <row r="11" spans="1:135">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -2994,8 +3203,19 @@
       <c r="DR11" s="1"/>
       <c r="DS11" s="1"/>
       <c r="DT11" s="1"/>
+      <c r="DU11" s="1"/>
+      <c r="DV11" s="1"/>
+      <c r="DW11" s="1"/>
+      <c r="DX11" s="1"/>
+      <c r="DY11" s="1"/>
+      <c r="DZ11" s="1"/>
+      <c r="EA11" s="1"/>
+      <c r="EB11" s="1"/>
+      <c r="EC11" s="1"/>
+      <c r="ED11" s="1"/>
+      <c r="EE11" s="1"/>
     </row>
-    <row r="12" spans="1:124">
+    <row r="12" spans="1:135">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -3120,8 +3340,19 @@
       <c r="DR12" s="1"/>
       <c r="DS12" s="1"/>
       <c r="DT12" s="1"/>
+      <c r="DU12" s="1"/>
+      <c r="DV12" s="1"/>
+      <c r="DW12" s="1"/>
+      <c r="DX12" s="1"/>
+      <c r="DY12" s="1"/>
+      <c r="DZ12" s="1"/>
+      <c r="EA12" s="1"/>
+      <c r="EB12" s="1"/>
+      <c r="EC12" s="1"/>
+      <c r="ED12" s="1"/>
+      <c r="EE12" s="1"/>
     </row>
-    <row r="13" spans="1:124">
+    <row r="13" spans="1:135">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -3246,8 +3477,19 @@
       <c r="DR13" s="1"/>
       <c r="DS13" s="1"/>
       <c r="DT13" s="1"/>
+      <c r="DU13" s="1"/>
+      <c r="DV13" s="1"/>
+      <c r="DW13" s="1"/>
+      <c r="DX13" s="1"/>
+      <c r="DY13" s="1"/>
+      <c r="DZ13" s="1"/>
+      <c r="EA13" s="1"/>
+      <c r="EB13" s="1"/>
+      <c r="EC13" s="1"/>
+      <c r="ED13" s="1"/>
+      <c r="EE13" s="1"/>
     </row>
-    <row r="14" spans="1:124">
+    <row r="14" spans="1:135">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -3372,8 +3614,19 @@
       <c r="DR14" s="1"/>
       <c r="DS14" s="1"/>
       <c r="DT14" s="1"/>
+      <c r="DU14" s="1"/>
+      <c r="DV14" s="1"/>
+      <c r="DW14" s="1"/>
+      <c r="DX14" s="1"/>
+      <c r="DY14" s="1"/>
+      <c r="DZ14" s="1"/>
+      <c r="EA14" s="1"/>
+      <c r="EB14" s="1"/>
+      <c r="EC14" s="1"/>
+      <c r="ED14" s="1"/>
+      <c r="EE14" s="1"/>
     </row>
-    <row r="15" spans="1:124">
+    <row r="15" spans="1:135">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -3498,8 +3751,19 @@
       <c r="DR15" s="1"/>
       <c r="DS15" s="1"/>
       <c r="DT15" s="1"/>
+      <c r="DU15" s="1"/>
+      <c r="DV15" s="1"/>
+      <c r="DW15" s="1"/>
+      <c r="DX15" s="1"/>
+      <c r="DY15" s="1"/>
+      <c r="DZ15" s="1"/>
+      <c r="EA15" s="1"/>
+      <c r="EB15" s="1"/>
+      <c r="EC15" s="1"/>
+      <c r="ED15" s="1"/>
+      <c r="EE15" s="1"/>
     </row>
-    <row r="16" spans="1:124">
+    <row r="16" spans="1:135">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -3624,8 +3888,19 @@
       <c r="DR16" s="1"/>
       <c r="DS16" s="1"/>
       <c r="DT16" s="1"/>
+      <c r="DU16" s="1"/>
+      <c r="DV16" s="1"/>
+      <c r="DW16" s="1"/>
+      <c r="DX16" s="1"/>
+      <c r="DY16" s="1"/>
+      <c r="DZ16" s="1"/>
+      <c r="EA16" s="1"/>
+      <c r="EB16" s="1"/>
+      <c r="EC16" s="1"/>
+      <c r="ED16" s="1"/>
+      <c r="EE16" s="1"/>
     </row>
-    <row r="17" spans="1:124">
+    <row r="17" spans="1:135">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -3750,8 +4025,19 @@
       <c r="DR17" s="1"/>
       <c r="DS17" s="1"/>
       <c r="DT17" s="1"/>
+      <c r="DU17" s="1"/>
+      <c r="DV17" s="1"/>
+      <c r="DW17" s="1"/>
+      <c r="DX17" s="1"/>
+      <c r="DY17" s="1"/>
+      <c r="DZ17" s="1"/>
+      <c r="EA17" s="1"/>
+      <c r="EB17" s="1"/>
+      <c r="EC17" s="1"/>
+      <c r="ED17" s="1"/>
+      <c r="EE17" s="1"/>
     </row>
-    <row r="18" spans="1:124">
+    <row r="18" spans="1:135">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -3876,8 +4162,19 @@
       <c r="DR18" s="1"/>
       <c r="DS18" s="1"/>
       <c r="DT18" s="1"/>
+      <c r="DU18" s="1"/>
+      <c r="DV18" s="1"/>
+      <c r="DW18" s="1"/>
+      <c r="DX18" s="1"/>
+      <c r="DY18" s="1"/>
+      <c r="DZ18" s="1"/>
+      <c r="EA18" s="1"/>
+      <c r="EB18" s="1"/>
+      <c r="EC18" s="1"/>
+      <c r="ED18" s="1"/>
+      <c r="EE18" s="1"/>
     </row>
-    <row r="19" spans="1:124">
+    <row r="19" spans="1:135">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -4002,8 +4299,19 @@
       <c r="DR19" s="1"/>
       <c r="DS19" s="1"/>
       <c r="DT19" s="1"/>
+      <c r="DU19" s="1"/>
+      <c r="DV19" s="1"/>
+      <c r="DW19" s="1"/>
+      <c r="DX19" s="1"/>
+      <c r="DY19" s="1"/>
+      <c r="DZ19" s="1"/>
+      <c r="EA19" s="1"/>
+      <c r="EB19" s="1"/>
+      <c r="EC19" s="1"/>
+      <c r="ED19" s="1"/>
+      <c r="EE19" s="1"/>
     </row>
-    <row r="20" spans="1:124">
+    <row r="20" spans="1:135">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -4128,8 +4436,19 @@
       <c r="DR20" s="1"/>
       <c r="DS20" s="1"/>
       <c r="DT20" s="1"/>
+      <c r="DU20" s="1"/>
+      <c r="DV20" s="1"/>
+      <c r="DW20" s="1"/>
+      <c r="DX20" s="1"/>
+      <c r="DY20" s="1"/>
+      <c r="DZ20" s="1"/>
+      <c r="EA20" s="1"/>
+      <c r="EB20" s="1"/>
+      <c r="EC20" s="1"/>
+      <c r="ED20" s="1"/>
+      <c r="EE20" s="1"/>
     </row>
-    <row r="21" spans="1:124">
+    <row r="21" spans="1:135">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -4254,8 +4573,19 @@
       <c r="DR21" s="1"/>
       <c r="DS21" s="1"/>
       <c r="DT21" s="1"/>
+      <c r="DU21" s="1"/>
+      <c r="DV21" s="1"/>
+      <c r="DW21" s="1"/>
+      <c r="DX21" s="1"/>
+      <c r="DY21" s="1"/>
+      <c r="DZ21" s="1"/>
+      <c r="EA21" s="1"/>
+      <c r="EB21" s="1"/>
+      <c r="EC21" s="1"/>
+      <c r="ED21" s="1"/>
+      <c r="EE21" s="1"/>
     </row>
-    <row r="22" spans="1:124">
+    <row r="22" spans="1:135">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -4380,8 +4710,19 @@
       <c r="DR22" s="1"/>
       <c r="DS22" s="1"/>
       <c r="DT22" s="1"/>
+      <c r="DU22" s="1"/>
+      <c r="DV22" s="1"/>
+      <c r="DW22" s="1"/>
+      <c r="DX22" s="1"/>
+      <c r="DY22" s="1"/>
+      <c r="DZ22" s="1"/>
+      <c r="EA22" s="1"/>
+      <c r="EB22" s="1"/>
+      <c r="EC22" s="1"/>
+      <c r="ED22" s="1"/>
+      <c r="EE22" s="1"/>
     </row>
-    <row r="23" spans="1:124">
+    <row r="23" spans="1:135">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -4506,8 +4847,19 @@
       <c r="DR23" s="1"/>
       <c r="DS23" s="1"/>
       <c r="DT23" s="1"/>
+      <c r="DU23" s="1"/>
+      <c r="DV23" s="1"/>
+      <c r="DW23" s="1"/>
+      <c r="DX23" s="1"/>
+      <c r="DY23" s="1"/>
+      <c r="DZ23" s="1"/>
+      <c r="EA23" s="1"/>
+      <c r="EB23" s="1"/>
+      <c r="EC23" s="1"/>
+      <c r="ED23" s="1"/>
+      <c r="EE23" s="1"/>
     </row>
-    <row r="24" spans="1:124">
+    <row r="24" spans="1:135">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -4632,8 +4984,19 @@
       <c r="DR24" s="1"/>
       <c r="DS24" s="1"/>
       <c r="DT24" s="1"/>
+      <c r="DU24" s="1"/>
+      <c r="DV24" s="1"/>
+      <c r="DW24" s="1"/>
+      <c r="DX24" s="1"/>
+      <c r="DY24" s="1"/>
+      <c r="DZ24" s="1"/>
+      <c r="EA24" s="1"/>
+      <c r="EB24" s="1"/>
+      <c r="EC24" s="1"/>
+      <c r="ED24" s="1"/>
+      <c r="EE24" s="1"/>
     </row>
-    <row r="25" spans="1:124">
+    <row r="25" spans="1:135">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -4758,8 +5121,19 @@
       <c r="DR25" s="1"/>
       <c r="DS25" s="1"/>
       <c r="DT25" s="1"/>
+      <c r="DU25" s="1"/>
+      <c r="DV25" s="1"/>
+      <c r="DW25" s="1"/>
+      <c r="DX25" s="1"/>
+      <c r="DY25" s="1"/>
+      <c r="DZ25" s="1"/>
+      <c r="EA25" s="1"/>
+      <c r="EB25" s="1"/>
+      <c r="EC25" s="1"/>
+      <c r="ED25" s="1"/>
+      <c r="EE25" s="1"/>
     </row>
-    <row r="26" spans="1:124">
+    <row r="26" spans="1:135">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -4884,8 +5258,19 @@
       <c r="DR26" s="1"/>
       <c r="DS26" s="1"/>
       <c r="DT26" s="1"/>
+      <c r="DU26" s="1"/>
+      <c r="DV26" s="1"/>
+      <c r="DW26" s="1"/>
+      <c r="DX26" s="1"/>
+      <c r="DY26" s="1"/>
+      <c r="DZ26" s="1"/>
+      <c r="EA26" s="1"/>
+      <c r="EB26" s="1"/>
+      <c r="EC26" s="1"/>
+      <c r="ED26" s="1"/>
+      <c r="EE26" s="1"/>
     </row>
-    <row r="27" spans="1:124">
+    <row r="27" spans="1:135">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -5010,8 +5395,19 @@
       <c r="DR27" s="1"/>
       <c r="DS27" s="1"/>
       <c r="DT27" s="1"/>
+      <c r="DU27" s="1"/>
+      <c r="DV27" s="1"/>
+      <c r="DW27" s="1"/>
+      <c r="DX27" s="1"/>
+      <c r="DY27" s="1"/>
+      <c r="DZ27" s="1"/>
+      <c r="EA27" s="1"/>
+      <c r="EB27" s="1"/>
+      <c r="EC27" s="1"/>
+      <c r="ED27" s="1"/>
+      <c r="EE27" s="1"/>
     </row>
-    <row r="28" spans="1:124">
+    <row r="28" spans="1:135">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -5136,8 +5532,19 @@
       <c r="DR28" s="1"/>
       <c r="DS28" s="1"/>
       <c r="DT28" s="1"/>
+      <c r="DU28" s="1"/>
+      <c r="DV28" s="1"/>
+      <c r="DW28" s="1"/>
+      <c r="DX28" s="1"/>
+      <c r="DY28" s="1"/>
+      <c r="DZ28" s="1"/>
+      <c r="EA28" s="1"/>
+      <c r="EB28" s="1"/>
+      <c r="EC28" s="1"/>
+      <c r="ED28" s="1"/>
+      <c r="EE28" s="1"/>
     </row>
-    <row r="29" spans="1:124">
+    <row r="29" spans="1:135">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -5262,8 +5669,19 @@
       <c r="DR29" s="1"/>
       <c r="DS29" s="1"/>
       <c r="DT29" s="1"/>
+      <c r="DU29" s="1"/>
+      <c r="DV29" s="1"/>
+      <c r="DW29" s="1"/>
+      <c r="DX29" s="1"/>
+      <c r="DY29" s="1"/>
+      <c r="DZ29" s="1"/>
+      <c r="EA29" s="1"/>
+      <c r="EB29" s="1"/>
+      <c r="EC29" s="1"/>
+      <c r="ED29" s="1"/>
+      <c r="EE29" s="1"/>
     </row>
-    <row r="30" spans="1:124">
+    <row r="30" spans="1:135">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -5388,8 +5806,19 @@
       <c r="DR30" s="1"/>
       <c r="DS30" s="1"/>
       <c r="DT30" s="1"/>
+      <c r="DU30" s="1"/>
+      <c r="DV30" s="1"/>
+      <c r="DW30" s="1"/>
+      <c r="DX30" s="1"/>
+      <c r="DY30" s="1"/>
+      <c r="DZ30" s="1"/>
+      <c r="EA30" s="1"/>
+      <c r="EB30" s="1"/>
+      <c r="EC30" s="1"/>
+      <c r="ED30" s="1"/>
+      <c r="EE30" s="1"/>
     </row>
-    <row r="31" spans="1:124">
+    <row r="31" spans="1:135">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -5514,8 +5943,19 @@
       <c r="DR31" s="1"/>
       <c r="DS31" s="1"/>
       <c r="DT31" s="1"/>
+      <c r="DU31" s="1"/>
+      <c r="DV31" s="1"/>
+      <c r="DW31" s="1"/>
+      <c r="DX31" s="1"/>
+      <c r="DY31" s="1"/>
+      <c r="DZ31" s="1"/>
+      <c r="EA31" s="1"/>
+      <c r="EB31" s="1"/>
+      <c r="EC31" s="1"/>
+      <c r="ED31" s="1"/>
+      <c r="EE31" s="1"/>
     </row>
-    <row r="32" spans="1:124">
+    <row r="32" spans="1:135">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -5640,8 +6080,19 @@
       <c r="DR32" s="1"/>
       <c r="DS32" s="1"/>
       <c r="DT32" s="1"/>
+      <c r="DU32" s="1"/>
+      <c r="DV32" s="1"/>
+      <c r="DW32" s="1"/>
+      <c r="DX32" s="1"/>
+      <c r="DY32" s="1"/>
+      <c r="DZ32" s="1"/>
+      <c r="EA32" s="1"/>
+      <c r="EB32" s="1"/>
+      <c r="EC32" s="1"/>
+      <c r="ED32" s="1"/>
+      <c r="EE32" s="1"/>
     </row>
-    <row r="33" spans="1:124">
+    <row r="33" spans="1:135">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -5766,8 +6217,19 @@
       <c r="DR33" s="1"/>
       <c r="DS33" s="1"/>
       <c r="DT33" s="1"/>
+      <c r="DU33" s="1"/>
+      <c r="DV33" s="1"/>
+      <c r="DW33" s="1"/>
+      <c r="DX33" s="1"/>
+      <c r="DY33" s="1"/>
+      <c r="DZ33" s="1"/>
+      <c r="EA33" s="1"/>
+      <c r="EB33" s="1"/>
+      <c r="EC33" s="1"/>
+      <c r="ED33" s="1"/>
+      <c r="EE33" s="1"/>
     </row>
-    <row r="34" spans="1:124">
+    <row r="34" spans="1:135">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -5892,8 +6354,19 @@
       <c r="DR34" s="1"/>
       <c r="DS34" s="1"/>
       <c r="DT34" s="1"/>
+      <c r="DU34" s="1"/>
+      <c r="DV34" s="1"/>
+      <c r="DW34" s="1"/>
+      <c r="DX34" s="1"/>
+      <c r="DY34" s="1"/>
+      <c r="DZ34" s="1"/>
+      <c r="EA34" s="1"/>
+      <c r="EB34" s="1"/>
+      <c r="EC34" s="1"/>
+      <c r="ED34" s="1"/>
+      <c r="EE34" s="1"/>
     </row>
-    <row r="35" spans="1:124">
+    <row r="35" spans="1:135">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -6018,8 +6491,19 @@
       <c r="DR35" s="1"/>
       <c r="DS35" s="1"/>
       <c r="DT35" s="1"/>
+      <c r="DU35" s="1"/>
+      <c r="DV35" s="1"/>
+      <c r="DW35" s="1"/>
+      <c r="DX35" s="1"/>
+      <c r="DY35" s="1"/>
+      <c r="DZ35" s="1"/>
+      <c r="EA35" s="1"/>
+      <c r="EB35" s="1"/>
+      <c r="EC35" s="1"/>
+      <c r="ED35" s="1"/>
+      <c r="EE35" s="1"/>
     </row>
-    <row r="36" spans="1:124">
+    <row r="36" spans="1:135">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -6144,8 +6628,19 @@
       <c r="DR36" s="1"/>
       <c r="DS36" s="1"/>
       <c r="DT36" s="1"/>
+      <c r="DU36" s="1"/>
+      <c r="DV36" s="1"/>
+      <c r="DW36" s="1"/>
+      <c r="DX36" s="1"/>
+      <c r="DY36" s="1"/>
+      <c r="DZ36" s="1"/>
+      <c r="EA36" s="1"/>
+      <c r="EB36" s="1"/>
+      <c r="EC36" s="1"/>
+      <c r="ED36" s="1"/>
+      <c r="EE36" s="1"/>
     </row>
-    <row r="37" spans="1:124">
+    <row r="37" spans="1:135">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -6270,8 +6765,19 @@
       <c r="DR37" s="1"/>
       <c r="DS37" s="1"/>
       <c r="DT37" s="1"/>
+      <c r="DU37" s="1"/>
+      <c r="DV37" s="1"/>
+      <c r="DW37" s="1"/>
+      <c r="DX37" s="1"/>
+      <c r="DY37" s="1"/>
+      <c r="DZ37" s="1"/>
+      <c r="EA37" s="1"/>
+      <c r="EB37" s="1"/>
+      <c r="EC37" s="1"/>
+      <c r="ED37" s="1"/>
+      <c r="EE37" s="1"/>
     </row>
-    <row r="38" spans="1:124">
+    <row r="38" spans="1:135">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -6396,8 +6902,19 @@
       <c r="DR38" s="1"/>
       <c r="DS38" s="1"/>
       <c r="DT38" s="1"/>
+      <c r="DU38" s="1"/>
+      <c r="DV38" s="1"/>
+      <c r="DW38" s="1"/>
+      <c r="DX38" s="1"/>
+      <c r="DY38" s="1"/>
+      <c r="DZ38" s="1"/>
+      <c r="EA38" s="1"/>
+      <c r="EB38" s="1"/>
+      <c r="EC38" s="1"/>
+      <c r="ED38" s="1"/>
+      <c r="EE38" s="1"/>
     </row>
-    <row r="39" spans="1:124">
+    <row r="39" spans="1:135">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -6522,8 +7039,19 @@
       <c r="DR39" s="1"/>
       <c r="DS39" s="1"/>
       <c r="DT39" s="1"/>
+      <c r="DU39" s="1"/>
+      <c r="DV39" s="1"/>
+      <c r="DW39" s="1"/>
+      <c r="DX39" s="1"/>
+      <c r="DY39" s="1"/>
+      <c r="DZ39" s="1"/>
+      <c r="EA39" s="1"/>
+      <c r="EB39" s="1"/>
+      <c r="EC39" s="1"/>
+      <c r="ED39" s="1"/>
+      <c r="EE39" s="1"/>
     </row>
-    <row r="40" spans="1:124">
+    <row r="40" spans="1:135">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -6648,8 +7176,19 @@
       <c r="DR40" s="1"/>
       <c r="DS40" s="1"/>
       <c r="DT40" s="1"/>
+      <c r="DU40" s="1"/>
+      <c r="DV40" s="1"/>
+      <c r="DW40" s="1"/>
+      <c r="DX40" s="1"/>
+      <c r="DY40" s="1"/>
+      <c r="DZ40" s="1"/>
+      <c r="EA40" s="1"/>
+      <c r="EB40" s="1"/>
+      <c r="EC40" s="1"/>
+      <c r="ED40" s="1"/>
+      <c r="EE40" s="1"/>
     </row>
-    <row r="41" spans="1:124">
+    <row r="41" spans="1:135">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -6774,8 +7313,19 @@
       <c r="DR41" s="1"/>
       <c r="DS41" s="1"/>
       <c r="DT41" s="1"/>
+      <c r="DU41" s="1"/>
+      <c r="DV41" s="1"/>
+      <c r="DW41" s="1"/>
+      <c r="DX41" s="1"/>
+      <c r="DY41" s="1"/>
+      <c r="DZ41" s="1"/>
+      <c r="EA41" s="1"/>
+      <c r="EB41" s="1"/>
+      <c r="EC41" s="1"/>
+      <c r="ED41" s="1"/>
+      <c r="EE41" s="1"/>
     </row>
-    <row r="42" spans="1:124">
+    <row r="42" spans="1:135">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -6900,8 +7450,19 @@
       <c r="DR42" s="1"/>
       <c r="DS42" s="1"/>
       <c r="DT42" s="1"/>
+      <c r="DU42" s="1"/>
+      <c r="DV42" s="1"/>
+      <c r="DW42" s="1"/>
+      <c r="DX42" s="1"/>
+      <c r="DY42" s="1"/>
+      <c r="DZ42" s="1"/>
+      <c r="EA42" s="1"/>
+      <c r="EB42" s="1"/>
+      <c r="EC42" s="1"/>
+      <c r="ED42" s="1"/>
+      <c r="EE42" s="1"/>
     </row>
-    <row r="43" spans="1:124">
+    <row r="43" spans="1:135">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -7026,8 +7587,19 @@
       <c r="DR43" s="1"/>
       <c r="DS43" s="1"/>
       <c r="DT43" s="1"/>
+      <c r="DU43" s="1"/>
+      <c r="DV43" s="1"/>
+      <c r="DW43" s="1"/>
+      <c r="DX43" s="1"/>
+      <c r="DY43" s="1"/>
+      <c r="DZ43" s="1"/>
+      <c r="EA43" s="1"/>
+      <c r="EB43" s="1"/>
+      <c r="EC43" s="1"/>
+      <c r="ED43" s="1"/>
+      <c r="EE43" s="1"/>
     </row>
-    <row r="44" spans="1:124">
+    <row r="44" spans="1:135">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -7152,8 +7724,19 @@
       <c r="DR44" s="1"/>
       <c r="DS44" s="1"/>
       <c r="DT44" s="1"/>
+      <c r="DU44" s="1"/>
+      <c r="DV44" s="1"/>
+      <c r="DW44" s="1"/>
+      <c r="DX44" s="1"/>
+      <c r="DY44" s="1"/>
+      <c r="DZ44" s="1"/>
+      <c r="EA44" s="1"/>
+      <c r="EB44" s="1"/>
+      <c r="EC44" s="1"/>
+      <c r="ED44" s="1"/>
+      <c r="EE44" s="1"/>
     </row>
-    <row r="45" spans="1:124">
+    <row r="45" spans="1:135">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -7278,8 +7861,19 @@
       <c r="DR45" s="1"/>
       <c r="DS45" s="1"/>
       <c r="DT45" s="1"/>
+      <c r="DU45" s="1"/>
+      <c r="DV45" s="1"/>
+      <c r="DW45" s="1"/>
+      <c r="DX45" s="1"/>
+      <c r="DY45" s="1"/>
+      <c r="DZ45" s="1"/>
+      <c r="EA45" s="1"/>
+      <c r="EB45" s="1"/>
+      <c r="EC45" s="1"/>
+      <c r="ED45" s="1"/>
+      <c r="EE45" s="1"/>
     </row>
-    <row r="46" spans="1:124">
+    <row r="46" spans="1:135">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -7404,8 +7998,19 @@
       <c r="DR46" s="1"/>
       <c r="DS46" s="1"/>
       <c r="DT46" s="1"/>
+      <c r="DU46" s="1"/>
+      <c r="DV46" s="1"/>
+      <c r="DW46" s="1"/>
+      <c r="DX46" s="1"/>
+      <c r="DY46" s="1"/>
+      <c r="DZ46" s="1"/>
+      <c r="EA46" s="1"/>
+      <c r="EB46" s="1"/>
+      <c r="EC46" s="1"/>
+      <c r="ED46" s="1"/>
+      <c r="EE46" s="1"/>
     </row>
-    <row r="47" spans="1:124">
+    <row r="47" spans="1:135">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -7530,8 +8135,19 @@
       <c r="DR47" s="1"/>
       <c r="DS47" s="1"/>
       <c r="DT47" s="1"/>
+      <c r="DU47" s="1"/>
+      <c r="DV47" s="1"/>
+      <c r="DW47" s="1"/>
+      <c r="DX47" s="1"/>
+      <c r="DY47" s="1"/>
+      <c r="DZ47" s="1"/>
+      <c r="EA47" s="1"/>
+      <c r="EB47" s="1"/>
+      <c r="EC47" s="1"/>
+      <c r="ED47" s="1"/>
+      <c r="EE47" s="1"/>
     </row>
-    <row r="48" spans="1:124">
+    <row r="48" spans="1:135">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -7656,8 +8272,19 @@
       <c r="DR48" s="1"/>
       <c r="DS48" s="1"/>
       <c r="DT48" s="1"/>
+      <c r="DU48" s="1"/>
+      <c r="DV48" s="1"/>
+      <c r="DW48" s="1"/>
+      <c r="DX48" s="1"/>
+      <c r="DY48" s="1"/>
+      <c r="DZ48" s="1"/>
+      <c r="EA48" s="1"/>
+      <c r="EB48" s="1"/>
+      <c r="EC48" s="1"/>
+      <c r="ED48" s="1"/>
+      <c r="EE48" s="1"/>
     </row>
-    <row r="49" spans="1:124">
+    <row r="49" spans="1:135">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -7782,8 +8409,19 @@
       <c r="DR49" s="1"/>
       <c r="DS49" s="1"/>
       <c r="DT49" s="1"/>
+      <c r="DU49" s="1"/>
+      <c r="DV49" s="1"/>
+      <c r="DW49" s="1"/>
+      <c r="DX49" s="1"/>
+      <c r="DY49" s="1"/>
+      <c r="DZ49" s="1"/>
+      <c r="EA49" s="1"/>
+      <c r="EB49" s="1"/>
+      <c r="EC49" s="1"/>
+      <c r="ED49" s="1"/>
+      <c r="EE49" s="1"/>
     </row>
-    <row r="50" spans="1:124">
+    <row r="50" spans="1:135">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -7908,8 +8546,19 @@
       <c r="DR50" s="1"/>
       <c r="DS50" s="1"/>
       <c r="DT50" s="1"/>
+      <c r="DU50" s="1"/>
+      <c r="DV50" s="1"/>
+      <c r="DW50" s="1"/>
+      <c r="DX50" s="1"/>
+      <c r="DY50" s="1"/>
+      <c r="DZ50" s="1"/>
+      <c r="EA50" s="1"/>
+      <c r="EB50" s="1"/>
+      <c r="EC50" s="1"/>
+      <c r="ED50" s="1"/>
+      <c r="EE50" s="1"/>
     </row>
-    <row r="51" spans="1:124">
+    <row r="51" spans="1:135">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -8034,8 +8683,19 @@
       <c r="DR51" s="1"/>
       <c r="DS51" s="1"/>
       <c r="DT51" s="1"/>
+      <c r="DU51" s="1"/>
+      <c r="DV51" s="1"/>
+      <c r="DW51" s="1"/>
+      <c r="DX51" s="1"/>
+      <c r="DY51" s="1"/>
+      <c r="DZ51" s="1"/>
+      <c r="EA51" s="1"/>
+      <c r="EB51" s="1"/>
+      <c r="EC51" s="1"/>
+      <c r="ED51" s="1"/>
+      <c r="EE51" s="1"/>
     </row>
-    <row r="52" spans="1:124">
+    <row r="52" spans="1:135">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -8160,8 +8820,19 @@
       <c r="DR52" s="1"/>
       <c r="DS52" s="1"/>
       <c r="DT52" s="1"/>
+      <c r="DU52" s="1"/>
+      <c r="DV52" s="1"/>
+      <c r="DW52" s="1"/>
+      <c r="DX52" s="1"/>
+      <c r="DY52" s="1"/>
+      <c r="DZ52" s="1"/>
+      <c r="EA52" s="1"/>
+      <c r="EB52" s="1"/>
+      <c r="EC52" s="1"/>
+      <c r="ED52" s="1"/>
+      <c r="EE52" s="1"/>
     </row>
-    <row r="53" spans="1:124">
+    <row r="53" spans="1:135">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -8286,8 +8957,19 @@
       <c r="DR53" s="1"/>
       <c r="DS53" s="1"/>
       <c r="DT53" s="1"/>
+      <c r="DU53" s="1"/>
+      <c r="DV53" s="1"/>
+      <c r="DW53" s="1"/>
+      <c r="DX53" s="1"/>
+      <c r="DY53" s="1"/>
+      <c r="DZ53" s="1"/>
+      <c r="EA53" s="1"/>
+      <c r="EB53" s="1"/>
+      <c r="EC53" s="1"/>
+      <c r="ED53" s="1"/>
+      <c r="EE53" s="1"/>
     </row>
-    <row r="54" spans="1:124">
+    <row r="54" spans="1:135">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -8412,8 +9094,19 @@
       <c r="DR54" s="1"/>
       <c r="DS54" s="1"/>
       <c r="DT54" s="1"/>
+      <c r="DU54" s="1"/>
+      <c r="DV54" s="1"/>
+      <c r="DW54" s="1"/>
+      <c r="DX54" s="1"/>
+      <c r="DY54" s="1"/>
+      <c r="DZ54" s="1"/>
+      <c r="EA54" s="1"/>
+      <c r="EB54" s="1"/>
+      <c r="EC54" s="1"/>
+      <c r="ED54" s="1"/>
+      <c r="EE54" s="1"/>
     </row>
-    <row r="55" spans="1:124">
+    <row r="55" spans="1:135">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -8538,8 +9231,19 @@
       <c r="DR55" s="1"/>
       <c r="DS55" s="1"/>
       <c r="DT55" s="1"/>
+      <c r="DU55" s="1"/>
+      <c r="DV55" s="1"/>
+      <c r="DW55" s="1"/>
+      <c r="DX55" s="1"/>
+      <c r="DY55" s="1"/>
+      <c r="DZ55" s="1"/>
+      <c r="EA55" s="1"/>
+      <c r="EB55" s="1"/>
+      <c r="EC55" s="1"/>
+      <c r="ED55" s="1"/>
+      <c r="EE55" s="1"/>
     </row>
-    <row r="56" spans="1:124">
+    <row r="56" spans="1:135">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -8664,8 +9368,19 @@
       <c r="DR56" s="1"/>
       <c r="DS56" s="1"/>
       <c r="DT56" s="1"/>
+      <c r="DU56" s="1"/>
+      <c r="DV56" s="1"/>
+      <c r="DW56" s="1"/>
+      <c r="DX56" s="1"/>
+      <c r="DY56" s="1"/>
+      <c r="DZ56" s="1"/>
+      <c r="EA56" s="1"/>
+      <c r="EB56" s="1"/>
+      <c r="EC56" s="1"/>
+      <c r="ED56" s="1"/>
+      <c r="EE56" s="1"/>
     </row>
-    <row r="57" spans="1:124">
+    <row r="57" spans="1:135">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -8790,8 +9505,19 @@
       <c r="DR57" s="1"/>
       <c r="DS57" s="1"/>
       <c r="DT57" s="1"/>
+      <c r="DU57" s="1"/>
+      <c r="DV57" s="1"/>
+      <c r="DW57" s="1"/>
+      <c r="DX57" s="1"/>
+      <c r="DY57" s="1"/>
+      <c r="DZ57" s="1"/>
+      <c r="EA57" s="1"/>
+      <c r="EB57" s="1"/>
+      <c r="EC57" s="1"/>
+      <c r="ED57" s="1"/>
+      <c r="EE57" s="1"/>
     </row>
-    <row r="58" spans="1:124">
+    <row r="58" spans="1:135">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -8916,8 +9642,19 @@
       <c r="DR58" s="1"/>
       <c r="DS58" s="1"/>
       <c r="DT58" s="1"/>
+      <c r="DU58" s="1"/>
+      <c r="DV58" s="1"/>
+      <c r="DW58" s="1"/>
+      <c r="DX58" s="1"/>
+      <c r="DY58" s="1"/>
+      <c r="DZ58" s="1"/>
+      <c r="EA58" s="1"/>
+      <c r="EB58" s="1"/>
+      <c r="EC58" s="1"/>
+      <c r="ED58" s="1"/>
+      <c r="EE58" s="1"/>
     </row>
-    <row r="59" spans="1:124">
+    <row r="59" spans="1:135">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -9042,8 +9779,19 @@
       <c r="DR59" s="1"/>
       <c r="DS59" s="1"/>
       <c r="DT59" s="1"/>
+      <c r="DU59" s="1"/>
+      <c r="DV59" s="1"/>
+      <c r="DW59" s="1"/>
+      <c r="DX59" s="1"/>
+      <c r="DY59" s="1"/>
+      <c r="DZ59" s="1"/>
+      <c r="EA59" s="1"/>
+      <c r="EB59" s="1"/>
+      <c r="EC59" s="1"/>
+      <c r="ED59" s="1"/>
+      <c r="EE59" s="1"/>
     </row>
-    <row r="60" spans="1:124">
+    <row r="60" spans="1:135">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -9168,8 +9916,19 @@
       <c r="DR60" s="1"/>
       <c r="DS60" s="1"/>
       <c r="DT60" s="1"/>
+      <c r="DU60" s="1"/>
+      <c r="DV60" s="1"/>
+      <c r="DW60" s="1"/>
+      <c r="DX60" s="1"/>
+      <c r="DY60" s="1"/>
+      <c r="DZ60" s="1"/>
+      <c r="EA60" s="1"/>
+      <c r="EB60" s="1"/>
+      <c r="EC60" s="1"/>
+      <c r="ED60" s="1"/>
+      <c r="EE60" s="1"/>
     </row>
-    <row r="61" spans="1:124">
+    <row r="61" spans="1:135">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -9294,8 +10053,19 @@
       <c r="DR61" s="1"/>
       <c r="DS61" s="1"/>
       <c r="DT61" s="1"/>
+      <c r="DU61" s="1"/>
+      <c r="DV61" s="1"/>
+      <c r="DW61" s="1"/>
+      <c r="DX61" s="1"/>
+      <c r="DY61" s="1"/>
+      <c r="DZ61" s="1"/>
+      <c r="EA61" s="1"/>
+      <c r="EB61" s="1"/>
+      <c r="EC61" s="1"/>
+      <c r="ED61" s="1"/>
+      <c r="EE61" s="1"/>
     </row>
-    <row r="62" spans="1:124">
+    <row r="62" spans="1:135">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -9420,8 +10190,19 @@
       <c r="DR62" s="1"/>
       <c r="DS62" s="1"/>
       <c r="DT62" s="1"/>
+      <c r="DU62" s="1"/>
+      <c r="DV62" s="1"/>
+      <c r="DW62" s="1"/>
+      <c r="DX62" s="1"/>
+      <c r="DY62" s="1"/>
+      <c r="DZ62" s="1"/>
+      <c r="EA62" s="1"/>
+      <c r="EB62" s="1"/>
+      <c r="EC62" s="1"/>
+      <c r="ED62" s="1"/>
+      <c r="EE62" s="1"/>
     </row>
-    <row r="63" spans="1:124">
+    <row r="63" spans="1:135">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -9546,8 +10327,19 @@
       <c r="DR63" s="1"/>
       <c r="DS63" s="1"/>
       <c r="DT63" s="1"/>
+      <c r="DU63" s="1"/>
+      <c r="DV63" s="1"/>
+      <c r="DW63" s="1"/>
+      <c r="DX63" s="1"/>
+      <c r="DY63" s="1"/>
+      <c r="DZ63" s="1"/>
+      <c r="EA63" s="1"/>
+      <c r="EB63" s="1"/>
+      <c r="EC63" s="1"/>
+      <c r="ED63" s="1"/>
+      <c r="EE63" s="1"/>
     </row>
-    <row r="64" spans="1:124">
+    <row r="64" spans="1:135">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -9672,8 +10464,19 @@
       <c r="DR64" s="1"/>
       <c r="DS64" s="1"/>
       <c r="DT64" s="1"/>
+      <c r="DU64" s="1"/>
+      <c r="DV64" s="1"/>
+      <c r="DW64" s="1"/>
+      <c r="DX64" s="1"/>
+      <c r="DY64" s="1"/>
+      <c r="DZ64" s="1"/>
+      <c r="EA64" s="1"/>
+      <c r="EB64" s="1"/>
+      <c r="EC64" s="1"/>
+      <c r="ED64" s="1"/>
+      <c r="EE64" s="1"/>
     </row>
-    <row r="65" spans="1:124">
+    <row r="65" spans="1:135">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -9798,8 +10601,19 @@
       <c r="DR65" s="1"/>
       <c r="DS65" s="1"/>
       <c r="DT65" s="1"/>
+      <c r="DU65" s="1"/>
+      <c r="DV65" s="1"/>
+      <c r="DW65" s="1"/>
+      <c r="DX65" s="1"/>
+      <c r="DY65" s="1"/>
+      <c r="DZ65" s="1"/>
+      <c r="EA65" s="1"/>
+      <c r="EB65" s="1"/>
+      <c r="EC65" s="1"/>
+      <c r="ED65" s="1"/>
+      <c r="EE65" s="1"/>
     </row>
-    <row r="66" spans="1:124">
+    <row r="66" spans="1:135">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -9924,8 +10738,19 @@
       <c r="DR66" s="1"/>
       <c r="DS66" s="1"/>
       <c r="DT66" s="1"/>
+      <c r="DU66" s="1"/>
+      <c r="DV66" s="1"/>
+      <c r="DW66" s="1"/>
+      <c r="DX66" s="1"/>
+      <c r="DY66" s="1"/>
+      <c r="DZ66" s="1"/>
+      <c r="EA66" s="1"/>
+      <c r="EB66" s="1"/>
+      <c r="EC66" s="1"/>
+      <c r="ED66" s="1"/>
+      <c r="EE66" s="1"/>
     </row>
-    <row r="67" spans="1:124">
+    <row r="67" spans="1:135">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -10050,8 +10875,19 @@
       <c r="DR67" s="1"/>
       <c r="DS67" s="1"/>
       <c r="DT67" s="1"/>
+      <c r="DU67" s="1"/>
+      <c r="DV67" s="1"/>
+      <c r="DW67" s="1"/>
+      <c r="DX67" s="1"/>
+      <c r="DY67" s="1"/>
+      <c r="DZ67" s="1"/>
+      <c r="EA67" s="1"/>
+      <c r="EB67" s="1"/>
+      <c r="EC67" s="1"/>
+      <c r="ED67" s="1"/>
+      <c r="EE67" s="1"/>
     </row>
-    <row r="68" spans="1:124">
+    <row r="68" spans="1:135">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -10176,8 +11012,19 @@
       <c r="DR68" s="1"/>
       <c r="DS68" s="1"/>
       <c r="DT68" s="1"/>
+      <c r="DU68" s="1"/>
+      <c r="DV68" s="1"/>
+      <c r="DW68" s="1"/>
+      <c r="DX68" s="1"/>
+      <c r="DY68" s="1"/>
+      <c r="DZ68" s="1"/>
+      <c r="EA68" s="1"/>
+      <c r="EB68" s="1"/>
+      <c r="EC68" s="1"/>
+      <c r="ED68" s="1"/>
+      <c r="EE68" s="1"/>
     </row>
-    <row r="69" spans="1:124">
+    <row r="69" spans="1:135">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -10302,8 +11149,19 @@
       <c r="DR69" s="1"/>
       <c r="DS69" s="1"/>
       <c r="DT69" s="1"/>
+      <c r="DU69" s="1"/>
+      <c r="DV69" s="1"/>
+      <c r="DW69" s="1"/>
+      <c r="DX69" s="1"/>
+      <c r="DY69" s="1"/>
+      <c r="DZ69" s="1"/>
+      <c r="EA69" s="1"/>
+      <c r="EB69" s="1"/>
+      <c r="EC69" s="1"/>
+      <c r="ED69" s="1"/>
+      <c r="EE69" s="1"/>
     </row>
-    <row r="70" spans="1:124">
+    <row r="70" spans="1:135">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -10428,8 +11286,19 @@
       <c r="DR70" s="1"/>
       <c r="DS70" s="1"/>
       <c r="DT70" s="1"/>
+      <c r="DU70" s="1"/>
+      <c r="DV70" s="1"/>
+      <c r="DW70" s="1"/>
+      <c r="DX70" s="1"/>
+      <c r="DY70" s="1"/>
+      <c r="DZ70" s="1"/>
+      <c r="EA70" s="1"/>
+      <c r="EB70" s="1"/>
+      <c r="EC70" s="1"/>
+      <c r="ED70" s="1"/>
+      <c r="EE70" s="1"/>
     </row>
-    <row r="71" spans="1:124">
+    <row r="71" spans="1:135">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -10554,8 +11423,19 @@
       <c r="DR71" s="1"/>
       <c r="DS71" s="1"/>
       <c r="DT71" s="1"/>
+      <c r="DU71" s="1"/>
+      <c r="DV71" s="1"/>
+      <c r="DW71" s="1"/>
+      <c r="DX71" s="1"/>
+      <c r="DY71" s="1"/>
+      <c r="DZ71" s="1"/>
+      <c r="EA71" s="1"/>
+      <c r="EB71" s="1"/>
+      <c r="EC71" s="1"/>
+      <c r="ED71" s="1"/>
+      <c r="EE71" s="1"/>
     </row>
-    <row r="72" spans="1:124">
+    <row r="72" spans="1:135">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -10680,8 +11560,19 @@
       <c r="DR72" s="1"/>
       <c r="DS72" s="1"/>
       <c r="DT72" s="1"/>
+      <c r="DU72" s="1"/>
+      <c r="DV72" s="1"/>
+      <c r="DW72" s="1"/>
+      <c r="DX72" s="1"/>
+      <c r="DY72" s="1"/>
+      <c r="DZ72" s="1"/>
+      <c r="EA72" s="1"/>
+      <c r="EB72" s="1"/>
+      <c r="EC72" s="1"/>
+      <c r="ED72" s="1"/>
+      <c r="EE72" s="1"/>
     </row>
-    <row r="73" spans="1:124">
+    <row r="73" spans="1:135">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -10806,8 +11697,19 @@
       <c r="DR73" s="1"/>
       <c r="DS73" s="1"/>
       <c r="DT73" s="1"/>
+      <c r="DU73" s="1"/>
+      <c r="DV73" s="1"/>
+      <c r="DW73" s="1"/>
+      <c r="DX73" s="1"/>
+      <c r="DY73" s="1"/>
+      <c r="DZ73" s="1"/>
+      <c r="EA73" s="1"/>
+      <c r="EB73" s="1"/>
+      <c r="EC73" s="1"/>
+      <c r="ED73" s="1"/>
+      <c r="EE73" s="1"/>
     </row>
-    <row r="74" spans="1:124">
+    <row r="74" spans="1:135">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -10932,8 +11834,19 @@
       <c r="DR74" s="1"/>
       <c r="DS74" s="1"/>
       <c r="DT74" s="1"/>
+      <c r="DU74" s="1"/>
+      <c r="DV74" s="1"/>
+      <c r="DW74" s="1"/>
+      <c r="DX74" s="1"/>
+      <c r="DY74" s="1"/>
+      <c r="DZ74" s="1"/>
+      <c r="EA74" s="1"/>
+      <c r="EB74" s="1"/>
+      <c r="EC74" s="1"/>
+      <c r="ED74" s="1"/>
+      <c r="EE74" s="1"/>
     </row>
-    <row r="75" spans="1:124">
+    <row r="75" spans="1:135">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -11058,8 +11971,19 @@
       <c r="DR75" s="1"/>
       <c r="DS75" s="1"/>
       <c r="DT75" s="1"/>
+      <c r="DU75" s="1"/>
+      <c r="DV75" s="1"/>
+      <c r="DW75" s="1"/>
+      <c r="DX75" s="1"/>
+      <c r="DY75" s="1"/>
+      <c r="DZ75" s="1"/>
+      <c r="EA75" s="1"/>
+      <c r="EB75" s="1"/>
+      <c r="EC75" s="1"/>
+      <c r="ED75" s="1"/>
+      <c r="EE75" s="1"/>
     </row>
-    <row r="76" spans="1:124">
+    <row r="76" spans="1:135">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -11184,8 +12108,19 @@
       <c r="DR76" s="1"/>
       <c r="DS76" s="1"/>
       <c r="DT76" s="1"/>
+      <c r="DU76" s="1"/>
+      <c r="DV76" s="1"/>
+      <c r="DW76" s="1"/>
+      <c r="DX76" s="1"/>
+      <c r="DY76" s="1"/>
+      <c r="DZ76" s="1"/>
+      <c r="EA76" s="1"/>
+      <c r="EB76" s="1"/>
+      <c r="EC76" s="1"/>
+      <c r="ED76" s="1"/>
+      <c r="EE76" s="1"/>
     </row>
-    <row r="77" spans="1:124">
+    <row r="77" spans="1:135">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -11310,8 +12245,19 @@
       <c r="DR77" s="1"/>
       <c r="DS77" s="1"/>
       <c r="DT77" s="1"/>
+      <c r="DU77" s="1"/>
+      <c r="DV77" s="1"/>
+      <c r="DW77" s="1"/>
+      <c r="DX77" s="1"/>
+      <c r="DY77" s="1"/>
+      <c r="DZ77" s="1"/>
+      <c r="EA77" s="1"/>
+      <c r="EB77" s="1"/>
+      <c r="EC77" s="1"/>
+      <c r="ED77" s="1"/>
+      <c r="EE77" s="1"/>
     </row>
-    <row r="78" spans="1:124">
+    <row r="78" spans="1:135">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -11436,8 +12382,19 @@
       <c r="DR78" s="1"/>
       <c r="DS78" s="1"/>
       <c r="DT78" s="1"/>
+      <c r="DU78" s="1"/>
+      <c r="DV78" s="1"/>
+      <c r="DW78" s="1"/>
+      <c r="DX78" s="1"/>
+      <c r="DY78" s="1"/>
+      <c r="DZ78" s="1"/>
+      <c r="EA78" s="1"/>
+      <c r="EB78" s="1"/>
+      <c r="EC78" s="1"/>
+      <c r="ED78" s="1"/>
+      <c r="EE78" s="1"/>
     </row>
-    <row r="79" spans="1:124">
+    <row r="79" spans="1:135">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -11562,8 +12519,19 @@
       <c r="DR79" s="1"/>
       <c r="DS79" s="1"/>
       <c r="DT79" s="1"/>
+      <c r="DU79" s="1"/>
+      <c r="DV79" s="1"/>
+      <c r="DW79" s="1"/>
+      <c r="DX79" s="1"/>
+      <c r="DY79" s="1"/>
+      <c r="DZ79" s="1"/>
+      <c r="EA79" s="1"/>
+      <c r="EB79" s="1"/>
+      <c r="EC79" s="1"/>
+      <c r="ED79" s="1"/>
+      <c r="EE79" s="1"/>
     </row>
-    <row r="80" spans="1:124">
+    <row r="80" spans="1:135">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -11688,8 +12656,19 @@
       <c r="DR80" s="1"/>
       <c r="DS80" s="1"/>
       <c r="DT80" s="1"/>
+      <c r="DU80" s="1"/>
+      <c r="DV80" s="1"/>
+      <c r="DW80" s="1"/>
+      <c r="DX80" s="1"/>
+      <c r="DY80" s="1"/>
+      <c r="DZ80" s="1"/>
+      <c r="EA80" s="1"/>
+      <c r="EB80" s="1"/>
+      <c r="EC80" s="1"/>
+      <c r="ED80" s="1"/>
+      <c r="EE80" s="1"/>
     </row>
-    <row r="81" spans="1:124">
+    <row r="81" spans="1:135">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -11814,8 +12793,19 @@
       <c r="DR81" s="1"/>
       <c r="DS81" s="1"/>
       <c r="DT81" s="1"/>
+      <c r="DU81" s="1"/>
+      <c r="DV81" s="1"/>
+      <c r="DW81" s="1"/>
+      <c r="DX81" s="1"/>
+      <c r="DY81" s="1"/>
+      <c r="DZ81" s="1"/>
+      <c r="EA81" s="1"/>
+      <c r="EB81" s="1"/>
+      <c r="EC81" s="1"/>
+      <c r="ED81" s="1"/>
+      <c r="EE81" s="1"/>
     </row>
-    <row r="82" spans="1:124">
+    <row r="82" spans="1:135">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -11940,8 +12930,19 @@
       <c r="DR82" s="1"/>
       <c r="DS82" s="1"/>
       <c r="DT82" s="1"/>
+      <c r="DU82" s="1"/>
+      <c r="DV82" s="1"/>
+      <c r="DW82" s="1"/>
+      <c r="DX82" s="1"/>
+      <c r="DY82" s="1"/>
+      <c r="DZ82" s="1"/>
+      <c r="EA82" s="1"/>
+      <c r="EB82" s="1"/>
+      <c r="EC82" s="1"/>
+      <c r="ED82" s="1"/>
+      <c r="EE82" s="1"/>
     </row>
-    <row r="83" spans="1:124">
+    <row r="83" spans="1:135">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -12066,8 +13067,19 @@
       <c r="DR83" s="1"/>
       <c r="DS83" s="1"/>
       <c r="DT83" s="1"/>
+      <c r="DU83" s="1"/>
+      <c r="DV83" s="1"/>
+      <c r="DW83" s="1"/>
+      <c r="DX83" s="1"/>
+      <c r="DY83" s="1"/>
+      <c r="DZ83" s="1"/>
+      <c r="EA83" s="1"/>
+      <c r="EB83" s="1"/>
+      <c r="EC83" s="1"/>
+      <c r="ED83" s="1"/>
+      <c r="EE83" s="1"/>
     </row>
-    <row r="84" spans="1:124">
+    <row r="84" spans="1:135">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -12192,8 +13204,19 @@
       <c r="DR84" s="1"/>
       <c r="DS84" s="1"/>
       <c r="DT84" s="1"/>
+      <c r="DU84" s="1"/>
+      <c r="DV84" s="1"/>
+      <c r="DW84" s="1"/>
+      <c r="DX84" s="1"/>
+      <c r="DY84" s="1"/>
+      <c r="DZ84" s="1"/>
+      <c r="EA84" s="1"/>
+      <c r="EB84" s="1"/>
+      <c r="EC84" s="1"/>
+      <c r="ED84" s="1"/>
+      <c r="EE84" s="1"/>
     </row>
-    <row r="85" spans="1:124">
+    <row r="85" spans="1:135">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -12318,8 +13341,19 @@
       <c r="DR85" s="1"/>
       <c r="DS85" s="1"/>
       <c r="DT85" s="1"/>
+      <c r="DU85" s="1"/>
+      <c r="DV85" s="1"/>
+      <c r="DW85" s="1"/>
+      <c r="DX85" s="1"/>
+      <c r="DY85" s="1"/>
+      <c r="DZ85" s="1"/>
+      <c r="EA85" s="1"/>
+      <c r="EB85" s="1"/>
+      <c r="EC85" s="1"/>
+      <c r="ED85" s="1"/>
+      <c r="EE85" s="1"/>
     </row>
-    <row r="86" spans="1:124">
+    <row r="86" spans="1:135">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -12444,8 +13478,19 @@
       <c r="DR86" s="1"/>
       <c r="DS86" s="1"/>
       <c r="DT86" s="1"/>
+      <c r="DU86" s="1"/>
+      <c r="DV86" s="1"/>
+      <c r="DW86" s="1"/>
+      <c r="DX86" s="1"/>
+      <c r="DY86" s="1"/>
+      <c r="DZ86" s="1"/>
+      <c r="EA86" s="1"/>
+      <c r="EB86" s="1"/>
+      <c r="EC86" s="1"/>
+      <c r="ED86" s="1"/>
+      <c r="EE86" s="1"/>
     </row>
-    <row r="87" spans="1:124">
+    <row r="87" spans="1:135">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -12570,8 +13615,19 @@
       <c r="DR87" s="1"/>
       <c r="DS87" s="1"/>
       <c r="DT87" s="1"/>
+      <c r="DU87" s="1"/>
+      <c r="DV87" s="1"/>
+      <c r="DW87" s="1"/>
+      <c r="DX87" s="1"/>
+      <c r="DY87" s="1"/>
+      <c r="DZ87" s="1"/>
+      <c r="EA87" s="1"/>
+      <c r="EB87" s="1"/>
+      <c r="EC87" s="1"/>
+      <c r="ED87" s="1"/>
+      <c r="EE87" s="1"/>
     </row>
-    <row r="88" spans="1:124">
+    <row r="88" spans="1:135">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -12696,8 +13752,19 @@
       <c r="DR88" s="1"/>
       <c r="DS88" s="1"/>
       <c r="DT88" s="1"/>
+      <c r="DU88" s="1"/>
+      <c r="DV88" s="1"/>
+      <c r="DW88" s="1"/>
+      <c r="DX88" s="1"/>
+      <c r="DY88" s="1"/>
+      <c r="DZ88" s="1"/>
+      <c r="EA88" s="1"/>
+      <c r="EB88" s="1"/>
+      <c r="EC88" s="1"/>
+      <c r="ED88" s="1"/>
+      <c r="EE88" s="1"/>
     </row>
-    <row r="89" spans="1:124">
+    <row r="89" spans="1:135">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -12822,8 +13889,19 @@
       <c r="DR89" s="1"/>
       <c r="DS89" s="1"/>
       <c r="DT89" s="1"/>
+      <c r="DU89" s="1"/>
+      <c r="DV89" s="1"/>
+      <c r="DW89" s="1"/>
+      <c r="DX89" s="1"/>
+      <c r="DY89" s="1"/>
+      <c r="DZ89" s="1"/>
+      <c r="EA89" s="1"/>
+      <c r="EB89" s="1"/>
+      <c r="EC89" s="1"/>
+      <c r="ED89" s="1"/>
+      <c r="EE89" s="1"/>
     </row>
-    <row r="90" spans="1:124">
+    <row r="90" spans="1:135">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
@@ -12948,8 +14026,19 @@
       <c r="DR90" s="1"/>
       <c r="DS90" s="1"/>
       <c r="DT90" s="1"/>
+      <c r="DU90" s="1"/>
+      <c r="DV90" s="1"/>
+      <c r="DW90" s="1"/>
+      <c r="DX90" s="1"/>
+      <c r="DY90" s="1"/>
+      <c r="DZ90" s="1"/>
+      <c r="EA90" s="1"/>
+      <c r="EB90" s="1"/>
+      <c r="EC90" s="1"/>
+      <c r="ED90" s="1"/>
+      <c r="EE90" s="1"/>
     </row>
-    <row r="91" spans="1:124">
+    <row r="91" spans="1:135">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -13074,8 +14163,19 @@
       <c r="DR91" s="1"/>
       <c r="DS91" s="1"/>
       <c r="DT91" s="1"/>
+      <c r="DU91" s="1"/>
+      <c r="DV91" s="1"/>
+      <c r="DW91" s="1"/>
+      <c r="DX91" s="1"/>
+      <c r="DY91" s="1"/>
+      <c r="DZ91" s="1"/>
+      <c r="EA91" s="1"/>
+      <c r="EB91" s="1"/>
+      <c r="EC91" s="1"/>
+      <c r="ED91" s="1"/>
+      <c r="EE91" s="1"/>
     </row>
-    <row r="92" spans="1:124">
+    <row r="92" spans="1:135">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -13200,8 +14300,19 @@
       <c r="DR92" s="1"/>
       <c r="DS92" s="1"/>
       <c r="DT92" s="1"/>
+      <c r="DU92" s="1"/>
+      <c r="DV92" s="1"/>
+      <c r="DW92" s="1"/>
+      <c r="DX92" s="1"/>
+      <c r="DY92" s="1"/>
+      <c r="DZ92" s="1"/>
+      <c r="EA92" s="1"/>
+      <c r="EB92" s="1"/>
+      <c r="EC92" s="1"/>
+      <c r="ED92" s="1"/>
+      <c r="EE92" s="1"/>
     </row>
-    <row r="93" spans="1:124">
+    <row r="93" spans="1:135">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -13326,8 +14437,19 @@
       <c r="DR93" s="1"/>
       <c r="DS93" s="1"/>
       <c r="DT93" s="1"/>
+      <c r="DU93" s="1"/>
+      <c r="DV93" s="1"/>
+      <c r="DW93" s="1"/>
+      <c r="DX93" s="1"/>
+      <c r="DY93" s="1"/>
+      <c r="DZ93" s="1"/>
+      <c r="EA93" s="1"/>
+      <c r="EB93" s="1"/>
+      <c r="EC93" s="1"/>
+      <c r="ED93" s="1"/>
+      <c r="EE93" s="1"/>
     </row>
-    <row r="94" spans="1:124">
+    <row r="94" spans="1:135">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -13452,8 +14574,19 @@
       <c r="DR94" s="1"/>
       <c r="DS94" s="1"/>
       <c r="DT94" s="1"/>
+      <c r="DU94" s="1"/>
+      <c r="DV94" s="1"/>
+      <c r="DW94" s="1"/>
+      <c r="DX94" s="1"/>
+      <c r="DY94" s="1"/>
+      <c r="DZ94" s="1"/>
+      <c r="EA94" s="1"/>
+      <c r="EB94" s="1"/>
+      <c r="EC94" s="1"/>
+      <c r="ED94" s="1"/>
+      <c r="EE94" s="1"/>
     </row>
-    <row r="95" spans="1:124">
+    <row r="95" spans="1:135">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -13578,8 +14711,19 @@
       <c r="DR95" s="1"/>
       <c r="DS95" s="1"/>
       <c r="DT95" s="1"/>
+      <c r="DU95" s="1"/>
+      <c r="DV95" s="1"/>
+      <c r="DW95" s="1"/>
+      <c r="DX95" s="1"/>
+      <c r="DY95" s="1"/>
+      <c r="DZ95" s="1"/>
+      <c r="EA95" s="1"/>
+      <c r="EB95" s="1"/>
+      <c r="EC95" s="1"/>
+      <c r="ED95" s="1"/>
+      <c r="EE95" s="1"/>
     </row>
-    <row r="96" spans="1:124">
+    <row r="96" spans="1:135">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -13704,8 +14848,19 @@
       <c r="DR96" s="1"/>
       <c r="DS96" s="1"/>
       <c r="DT96" s="1"/>
+      <c r="DU96" s="1"/>
+      <c r="DV96" s="1"/>
+      <c r="DW96" s="1"/>
+      <c r="DX96" s="1"/>
+      <c r="DY96" s="1"/>
+      <c r="DZ96" s="1"/>
+      <c r="EA96" s="1"/>
+      <c r="EB96" s="1"/>
+      <c r="EC96" s="1"/>
+      <c r="ED96" s="1"/>
+      <c r="EE96" s="1"/>
     </row>
-    <row r="97" spans="1:124">
+    <row r="97" spans="1:135">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
@@ -13830,8 +14985,19 @@
       <c r="DR97" s="1"/>
       <c r="DS97" s="1"/>
       <c r="DT97" s="1"/>
+      <c r="DU97" s="1"/>
+      <c r="DV97" s="1"/>
+      <c r="DW97" s="1"/>
+      <c r="DX97" s="1"/>
+      <c r="DY97" s="1"/>
+      <c r="DZ97" s="1"/>
+      <c r="EA97" s="1"/>
+      <c r="EB97" s="1"/>
+      <c r="EC97" s="1"/>
+      <c r="ED97" s="1"/>
+      <c r="EE97" s="1"/>
     </row>
-    <row r="98" spans="1:124">
+    <row r="98" spans="1:135">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -13956,8 +15122,19 @@
       <c r="DR98" s="1"/>
       <c r="DS98" s="1"/>
       <c r="DT98" s="1"/>
+      <c r="DU98" s="1"/>
+      <c r="DV98" s="1"/>
+      <c r="DW98" s="1"/>
+      <c r="DX98" s="1"/>
+      <c r="DY98" s="1"/>
+      <c r="DZ98" s="1"/>
+      <c r="EA98" s="1"/>
+      <c r="EB98" s="1"/>
+      <c r="EC98" s="1"/>
+      <c r="ED98" s="1"/>
+      <c r="EE98" s="1"/>
     </row>
-    <row r="99" spans="1:124">
+    <row r="99" spans="1:135">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
@@ -14082,8 +15259,19 @@
       <c r="DR99" s="1"/>
       <c r="DS99" s="1"/>
       <c r="DT99" s="1"/>
+      <c r="DU99" s="1"/>
+      <c r="DV99" s="1"/>
+      <c r="DW99" s="1"/>
+      <c r="DX99" s="1"/>
+      <c r="DY99" s="1"/>
+      <c r="DZ99" s="1"/>
+      <c r="EA99" s="1"/>
+      <c r="EB99" s="1"/>
+      <c r="EC99" s="1"/>
+      <c r="ED99" s="1"/>
+      <c r="EE99" s="1"/>
     </row>
-    <row r="100" spans="1:124">
+    <row r="100" spans="1:135">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
@@ -14208,8 +15396,19 @@
       <c r="DR100" s="1"/>
       <c r="DS100" s="1"/>
       <c r="DT100" s="1"/>
+      <c r="DU100" s="1"/>
+      <c r="DV100" s="1"/>
+      <c r="DW100" s="1"/>
+      <c r="DX100" s="1"/>
+      <c r="DY100" s="1"/>
+      <c r="DZ100" s="1"/>
+      <c r="EA100" s="1"/>
+      <c r="EB100" s="1"/>
+      <c r="EC100" s="1"/>
+      <c r="ED100" s="1"/>
+      <c r="EE100" s="1"/>
     </row>
-    <row r="101" spans="1:124">
+    <row r="101" spans="1:135">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
@@ -14334,8 +15533,19 @@
       <c r="DR101" s="1"/>
       <c r="DS101" s="1"/>
       <c r="DT101" s="1"/>
+      <c r="DU101" s="1"/>
+      <c r="DV101" s="1"/>
+      <c r="DW101" s="1"/>
+      <c r="DX101" s="1"/>
+      <c r="DY101" s="1"/>
+      <c r="DZ101" s="1"/>
+      <c r="EA101" s="1"/>
+      <c r="EB101" s="1"/>
+      <c r="EC101" s="1"/>
+      <c r="ED101" s="1"/>
+      <c r="EE101" s="1"/>
     </row>
-    <row r="102" spans="1:124">
+    <row r="102" spans="1:135">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -14460,8 +15670,19 @@
       <c r="DR102" s="1"/>
       <c r="DS102" s="1"/>
       <c r="DT102" s="1"/>
+      <c r="DU102" s="1"/>
+      <c r="DV102" s="1"/>
+      <c r="DW102" s="1"/>
+      <c r="DX102" s="1"/>
+      <c r="DY102" s="1"/>
+      <c r="DZ102" s="1"/>
+      <c r="EA102" s="1"/>
+      <c r="EB102" s="1"/>
+      <c r="EC102" s="1"/>
+      <c r="ED102" s="1"/>
+      <c r="EE102" s="1"/>
     </row>
-    <row r="103" spans="1:124">
+    <row r="103" spans="1:135">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -14586,8 +15807,19 @@
       <c r="DR103" s="1"/>
       <c r="DS103" s="1"/>
       <c r="DT103" s="1"/>
+      <c r="DU103" s="1"/>
+      <c r="DV103" s="1"/>
+      <c r="DW103" s="1"/>
+      <c r="DX103" s="1"/>
+      <c r="DY103" s="1"/>
+      <c r="DZ103" s="1"/>
+      <c r="EA103" s="1"/>
+      <c r="EB103" s="1"/>
+      <c r="EC103" s="1"/>
+      <c r="ED103" s="1"/>
+      <c r="EE103" s="1"/>
     </row>
-    <row r="104" spans="1:124">
+    <row r="104" spans="1:135">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -14712,8 +15944,19 @@
       <c r="DR104" s="1"/>
       <c r="DS104" s="1"/>
       <c r="DT104" s="1"/>
+      <c r="DU104" s="1"/>
+      <c r="DV104" s="1"/>
+      <c r="DW104" s="1"/>
+      <c r="DX104" s="1"/>
+      <c r="DY104" s="1"/>
+      <c r="DZ104" s="1"/>
+      <c r="EA104" s="1"/>
+      <c r="EB104" s="1"/>
+      <c r="EC104" s="1"/>
+      <c r="ED104" s="1"/>
+      <c r="EE104" s="1"/>
     </row>
-    <row r="105" spans="1:124">
+    <row r="105" spans="1:135">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
@@ -14838,8 +16081,19 @@
       <c r="DR105" s="1"/>
       <c r="DS105" s="1"/>
       <c r="DT105" s="1"/>
+      <c r="DU105" s="1"/>
+      <c r="DV105" s="1"/>
+      <c r="DW105" s="1"/>
+      <c r="DX105" s="1"/>
+      <c r="DY105" s="1"/>
+      <c r="DZ105" s="1"/>
+      <c r="EA105" s="1"/>
+      <c r="EB105" s="1"/>
+      <c r="EC105" s="1"/>
+      <c r="ED105" s="1"/>
+      <c r="EE105" s="1"/>
     </row>
-    <row r="106" spans="1:124">
+    <row r="106" spans="1:135">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
@@ -14964,8 +16218,19 @@
       <c r="DR106" s="1"/>
       <c r="DS106" s="1"/>
       <c r="DT106" s="1"/>
+      <c r="DU106" s="1"/>
+      <c r="DV106" s="1"/>
+      <c r="DW106" s="1"/>
+      <c r="DX106" s="1"/>
+      <c r="DY106" s="1"/>
+      <c r="DZ106" s="1"/>
+      <c r="EA106" s="1"/>
+      <c r="EB106" s="1"/>
+      <c r="EC106" s="1"/>
+      <c r="ED106" s="1"/>
+      <c r="EE106" s="1"/>
     </row>
-    <row r="107" spans="1:124">
+    <row r="107" spans="1:135">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
@@ -15090,8 +16355,19 @@
       <c r="DR107" s="1"/>
       <c r="DS107" s="1"/>
       <c r="DT107" s="1"/>
+      <c r="DU107" s="1"/>
+      <c r="DV107" s="1"/>
+      <c r="DW107" s="1"/>
+      <c r="DX107" s="1"/>
+      <c r="DY107" s="1"/>
+      <c r="DZ107" s="1"/>
+      <c r="EA107" s="1"/>
+      <c r="EB107" s="1"/>
+      <c r="EC107" s="1"/>
+      <c r="ED107" s="1"/>
+      <c r="EE107" s="1"/>
     </row>
-    <row r="108" spans="1:124">
+    <row r="108" spans="1:135">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
@@ -15216,8 +16492,19 @@
       <c r="DR108" s="1"/>
       <c r="DS108" s="1"/>
       <c r="DT108" s="1"/>
+      <c r="DU108" s="1"/>
+      <c r="DV108" s="1"/>
+      <c r="DW108" s="1"/>
+      <c r="DX108" s="1"/>
+      <c r="DY108" s="1"/>
+      <c r="DZ108" s="1"/>
+      <c r="EA108" s="1"/>
+      <c r="EB108" s="1"/>
+      <c r="EC108" s="1"/>
+      <c r="ED108" s="1"/>
+      <c r="EE108" s="1"/>
     </row>
-    <row r="109" spans="1:124">
+    <row r="109" spans="1:135">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -15342,8 +16629,19 @@
       <c r="DR109" s="1"/>
       <c r="DS109" s="1"/>
       <c r="DT109" s="1"/>
+      <c r="DU109" s="1"/>
+      <c r="DV109" s="1"/>
+      <c r="DW109" s="1"/>
+      <c r="DX109" s="1"/>
+      <c r="DY109" s="1"/>
+      <c r="DZ109" s="1"/>
+      <c r="EA109" s="1"/>
+      <c r="EB109" s="1"/>
+      <c r="EC109" s="1"/>
+      <c r="ED109" s="1"/>
+      <c r="EE109" s="1"/>
     </row>
-    <row r="110" spans="1:124">
+    <row r="110" spans="1:135">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -15468,8 +16766,19 @@
       <c r="DR110" s="1"/>
       <c r="DS110" s="1"/>
       <c r="DT110" s="1"/>
+      <c r="DU110" s="1"/>
+      <c r="DV110" s="1"/>
+      <c r="DW110" s="1"/>
+      <c r="DX110" s="1"/>
+      <c r="DY110" s="1"/>
+      <c r="DZ110" s="1"/>
+      <c r="EA110" s="1"/>
+      <c r="EB110" s="1"/>
+      <c r="EC110" s="1"/>
+      <c r="ED110" s="1"/>
+      <c r="EE110" s="1"/>
     </row>
-    <row r="111" spans="1:124">
+    <row r="111" spans="1:135">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
@@ -15594,8 +16903,19 @@
       <c r="DR111" s="1"/>
       <c r="DS111" s="1"/>
       <c r="DT111" s="1"/>
+      <c r="DU111" s="1"/>
+      <c r="DV111" s="1"/>
+      <c r="DW111" s="1"/>
+      <c r="DX111" s="1"/>
+      <c r="DY111" s="1"/>
+      <c r="DZ111" s="1"/>
+      <c r="EA111" s="1"/>
+      <c r="EB111" s="1"/>
+      <c r="EC111" s="1"/>
+      <c r="ED111" s="1"/>
+      <c r="EE111" s="1"/>
     </row>
-    <row r="112" spans="1:124">
+    <row r="112" spans="1:135">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
@@ -15720,8 +17040,19 @@
       <c r="DR112" s="1"/>
       <c r="DS112" s="1"/>
       <c r="DT112" s="1"/>
+      <c r="DU112" s="1"/>
+      <c r="DV112" s="1"/>
+      <c r="DW112" s="1"/>
+      <c r="DX112" s="1"/>
+      <c r="DY112" s="1"/>
+      <c r="DZ112" s="1"/>
+      <c r="EA112" s="1"/>
+      <c r="EB112" s="1"/>
+      <c r="EC112" s="1"/>
+      <c r="ED112" s="1"/>
+      <c r="EE112" s="1"/>
     </row>
-    <row r="113" spans="1:124">
+    <row r="113" spans="1:135">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
@@ -15846,8 +17177,19 @@
       <c r="DR113" s="1"/>
       <c r="DS113" s="1"/>
       <c r="DT113" s="1"/>
+      <c r="DU113" s="1"/>
+      <c r="DV113" s="1"/>
+      <c r="DW113" s="1"/>
+      <c r="DX113" s="1"/>
+      <c r="DY113" s="1"/>
+      <c r="DZ113" s="1"/>
+      <c r="EA113" s="1"/>
+      <c r="EB113" s="1"/>
+      <c r="EC113" s="1"/>
+      <c r="ED113" s="1"/>
+      <c r="EE113" s="1"/>
     </row>
-    <row r="114" spans="1:124">
+    <row r="114" spans="1:135">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -15972,8 +17314,19 @@
       <c r="DR114" s="1"/>
       <c r="DS114" s="1"/>
       <c r="DT114" s="1"/>
+      <c r="DU114" s="1"/>
+      <c r="DV114" s="1"/>
+      <c r="DW114" s="1"/>
+      <c r="DX114" s="1"/>
+      <c r="DY114" s="1"/>
+      <c r="DZ114" s="1"/>
+      <c r="EA114" s="1"/>
+      <c r="EB114" s="1"/>
+      <c r="EC114" s="1"/>
+      <c r="ED114" s="1"/>
+      <c r="EE114" s="1"/>
     </row>
-    <row r="115" spans="1:124">
+    <row r="115" spans="1:135">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
@@ -16098,8 +17451,19 @@
       <c r="DR115" s="1"/>
       <c r="DS115" s="1"/>
       <c r="DT115" s="1"/>
+      <c r="DU115" s="1"/>
+      <c r="DV115" s="1"/>
+      <c r="DW115" s="1"/>
+      <c r="DX115" s="1"/>
+      <c r="DY115" s="1"/>
+      <c r="DZ115" s="1"/>
+      <c r="EA115" s="1"/>
+      <c r="EB115" s="1"/>
+      <c r="EC115" s="1"/>
+      <c r="ED115" s="1"/>
+      <c r="EE115" s="1"/>
     </row>
-    <row r="116" spans="1:124">
+    <row r="116" spans="1:135">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -16224,8 +17588,19 @@
       <c r="DR116" s="1"/>
       <c r="DS116" s="1"/>
       <c r="DT116" s="1"/>
+      <c r="DU116" s="1"/>
+      <c r="DV116" s="1"/>
+      <c r="DW116" s="1"/>
+      <c r="DX116" s="1"/>
+      <c r="DY116" s="1"/>
+      <c r="DZ116" s="1"/>
+      <c r="EA116" s="1"/>
+      <c r="EB116" s="1"/>
+      <c r="EC116" s="1"/>
+      <c r="ED116" s="1"/>
+      <c r="EE116" s="1"/>
     </row>
-    <row r="117" spans="1:124">
+    <row r="117" spans="1:135">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
@@ -16350,8 +17725,19 @@
       <c r="DR117" s="1"/>
       <c r="DS117" s="1"/>
       <c r="DT117" s="1"/>
+      <c r="DU117" s="1"/>
+      <c r="DV117" s="1"/>
+      <c r="DW117" s="1"/>
+      <c r="DX117" s="1"/>
+      <c r="DY117" s="1"/>
+      <c r="DZ117" s="1"/>
+      <c r="EA117" s="1"/>
+      <c r="EB117" s="1"/>
+      <c r="EC117" s="1"/>
+      <c r="ED117" s="1"/>
+      <c r="EE117" s="1"/>
     </row>
-    <row r="118" spans="1:124">
+    <row r="118" spans="1:135">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
@@ -16476,8 +17862,19 @@
       <c r="DR118" s="1"/>
       <c r="DS118" s="1"/>
       <c r="DT118" s="1"/>
+      <c r="DU118" s="1"/>
+      <c r="DV118" s="1"/>
+      <c r="DW118" s="1"/>
+      <c r="DX118" s="1"/>
+      <c r="DY118" s="1"/>
+      <c r="DZ118" s="1"/>
+      <c r="EA118" s="1"/>
+      <c r="EB118" s="1"/>
+      <c r="EC118" s="1"/>
+      <c r="ED118" s="1"/>
+      <c r="EE118" s="1"/>
     </row>
-    <row r="119" spans="1:124">
+    <row r="119" spans="1:135">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
@@ -16602,8 +17999,19 @@
       <c r="DR119" s="1"/>
       <c r="DS119" s="1"/>
       <c r="DT119" s="1"/>
+      <c r="DU119" s="1"/>
+      <c r="DV119" s="1"/>
+      <c r="DW119" s="1"/>
+      <c r="DX119" s="1"/>
+      <c r="DY119" s="1"/>
+      <c r="DZ119" s="1"/>
+      <c r="EA119" s="1"/>
+      <c r="EB119" s="1"/>
+      <c r="EC119" s="1"/>
+      <c r="ED119" s="1"/>
+      <c r="EE119" s="1"/>
     </row>
-    <row r="120" spans="1:124">
+    <row r="120" spans="1:135">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
@@ -16728,8 +18136,19 @@
       <c r="DR120" s="1"/>
       <c r="DS120" s="1"/>
       <c r="DT120" s="1"/>
+      <c r="DU120" s="1"/>
+      <c r="DV120" s="1"/>
+      <c r="DW120" s="1"/>
+      <c r="DX120" s="1"/>
+      <c r="DY120" s="1"/>
+      <c r="DZ120" s="1"/>
+      <c r="EA120" s="1"/>
+      <c r="EB120" s="1"/>
+      <c r="EC120" s="1"/>
+      <c r="ED120" s="1"/>
+      <c r="EE120" s="1"/>
     </row>
-    <row r="121" spans="1:124">
+    <row r="121" spans="1:135">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
@@ -16854,8 +18273,19 @@
       <c r="DR121" s="1"/>
       <c r="DS121" s="1"/>
       <c r="DT121" s="1"/>
+      <c r="DU121" s="1"/>
+      <c r="DV121" s="1"/>
+      <c r="DW121" s="1"/>
+      <c r="DX121" s="1"/>
+      <c r="DY121" s="1"/>
+      <c r="DZ121" s="1"/>
+      <c r="EA121" s="1"/>
+      <c r="EB121" s="1"/>
+      <c r="EC121" s="1"/>
+      <c r="ED121" s="1"/>
+      <c r="EE121" s="1"/>
     </row>
-    <row r="122" spans="1:124">
+    <row r="122" spans="1:135">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -16980,8 +18410,19 @@
       <c r="DR122" s="1"/>
       <c r="DS122" s="1"/>
       <c r="DT122" s="1"/>
+      <c r="DU122" s="1"/>
+      <c r="DV122" s="1"/>
+      <c r="DW122" s="1"/>
+      <c r="DX122" s="1"/>
+      <c r="DY122" s="1"/>
+      <c r="DZ122" s="1"/>
+      <c r="EA122" s="1"/>
+      <c r="EB122" s="1"/>
+      <c r="EC122" s="1"/>
+      <c r="ED122" s="1"/>
+      <c r="EE122" s="1"/>
     </row>
-    <row r="123" spans="1:124">
+    <row r="123" spans="1:135">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
@@ -17106,8 +18547,19 @@
       <c r="DR123" s="1"/>
       <c r="DS123" s="1"/>
       <c r="DT123" s="1"/>
+      <c r="DU123" s="1"/>
+      <c r="DV123" s="1"/>
+      <c r="DW123" s="1"/>
+      <c r="DX123" s="1"/>
+      <c r="DY123" s="1"/>
+      <c r="DZ123" s="1"/>
+      <c r="EA123" s="1"/>
+      <c r="EB123" s="1"/>
+      <c r="EC123" s="1"/>
+      <c r="ED123" s="1"/>
+      <c r="EE123" s="1"/>
     </row>
-    <row r="124" spans="1:124">
+    <row r="124" spans="1:135">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
@@ -17232,8 +18684,19 @@
       <c r="DR124" s="1"/>
       <c r="DS124" s="1"/>
       <c r="DT124" s="1"/>
+      <c r="DU124" s="1"/>
+      <c r="DV124" s="1"/>
+      <c r="DW124" s="1"/>
+      <c r="DX124" s="1"/>
+      <c r="DY124" s="1"/>
+      <c r="DZ124" s="1"/>
+      <c r="EA124" s="1"/>
+      <c r="EB124" s="1"/>
+      <c r="EC124" s="1"/>
+      <c r="ED124" s="1"/>
+      <c r="EE124" s="1"/>
     </row>
-    <row r="125" spans="1:124">
+    <row r="125" spans="1:135">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
@@ -17358,8 +18821,19 @@
       <c r="DR125" s="1"/>
       <c r="DS125" s="1"/>
       <c r="DT125" s="1"/>
+      <c r="DU125" s="1"/>
+      <c r="DV125" s="1"/>
+      <c r="DW125" s="1"/>
+      <c r="DX125" s="1"/>
+      <c r="DY125" s="1"/>
+      <c r="DZ125" s="1"/>
+      <c r="EA125" s="1"/>
+      <c r="EB125" s="1"/>
+      <c r="EC125" s="1"/>
+      <c r="ED125" s="1"/>
+      <c r="EE125" s="1"/>
     </row>
-    <row r="126" spans="1:124">
+    <row r="126" spans="1:135">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
@@ -17484,8 +18958,19 @@
       <c r="DR126" s="1"/>
       <c r="DS126" s="1"/>
       <c r="DT126" s="1"/>
+      <c r="DU126" s="1"/>
+      <c r="DV126" s="1"/>
+      <c r="DW126" s="1"/>
+      <c r="DX126" s="1"/>
+      <c r="DY126" s="1"/>
+      <c r="DZ126" s="1"/>
+      <c r="EA126" s="1"/>
+      <c r="EB126" s="1"/>
+      <c r="EC126" s="1"/>
+      <c r="ED126" s="1"/>
+      <c r="EE126" s="1"/>
     </row>
-    <row r="127" spans="1:124">
+    <row r="127" spans="1:135">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
@@ -17610,8 +19095,19 @@
       <c r="DR127" s="1"/>
       <c r="DS127" s="1"/>
       <c r="DT127" s="1"/>
+      <c r="DU127" s="1"/>
+      <c r="DV127" s="1"/>
+      <c r="DW127" s="1"/>
+      <c r="DX127" s="1"/>
+      <c r="DY127" s="1"/>
+      <c r="DZ127" s="1"/>
+      <c r="EA127" s="1"/>
+      <c r="EB127" s="1"/>
+      <c r="EC127" s="1"/>
+      <c r="ED127" s="1"/>
+      <c r="EE127" s="1"/>
     </row>
-    <row r="128" spans="1:124">
+    <row r="128" spans="1:135">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
@@ -17736,8 +19232,19 @@
       <c r="DR128" s="1"/>
       <c r="DS128" s="1"/>
       <c r="DT128" s="1"/>
+      <c r="DU128" s="1"/>
+      <c r="DV128" s="1"/>
+      <c r="DW128" s="1"/>
+      <c r="DX128" s="1"/>
+      <c r="DY128" s="1"/>
+      <c r="DZ128" s="1"/>
+      <c r="EA128" s="1"/>
+      <c r="EB128" s="1"/>
+      <c r="EC128" s="1"/>
+      <c r="ED128" s="1"/>
+      <c r="EE128" s="1"/>
     </row>
-    <row r="129" spans="1:124">
+    <row r="129" spans="1:135">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
@@ -17862,8 +19369,19 @@
       <c r="DR129" s="1"/>
       <c r="DS129" s="1"/>
       <c r="DT129" s="1"/>
+      <c r="DU129" s="1"/>
+      <c r="DV129" s="1"/>
+      <c r="DW129" s="1"/>
+      <c r="DX129" s="1"/>
+      <c r="DY129" s="1"/>
+      <c r="DZ129" s="1"/>
+      <c r="EA129" s="1"/>
+      <c r="EB129" s="1"/>
+      <c r="EC129" s="1"/>
+      <c r="ED129" s="1"/>
+      <c r="EE129" s="1"/>
     </row>
-    <row r="130" spans="1:124">
+    <row r="130" spans="1:135">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
@@ -17988,8 +19506,19 @@
       <c r="DR130" s="1"/>
       <c r="DS130" s="1"/>
       <c r="DT130" s="1"/>
+      <c r="DU130" s="1"/>
+      <c r="DV130" s="1"/>
+      <c r="DW130" s="1"/>
+      <c r="DX130" s="1"/>
+      <c r="DY130" s="1"/>
+      <c r="DZ130" s="1"/>
+      <c r="EA130" s="1"/>
+      <c r="EB130" s="1"/>
+      <c r="EC130" s="1"/>
+      <c r="ED130" s="1"/>
+      <c r="EE130" s="1"/>
     </row>
-    <row r="131" spans="1:124">
+    <row r="131" spans="1:135">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
@@ -18114,8 +19643,19 @@
       <c r="DR131" s="1"/>
       <c r="DS131" s="1"/>
       <c r="DT131" s="1"/>
+      <c r="DU131" s="1"/>
+      <c r="DV131" s="1"/>
+      <c r="DW131" s="1"/>
+      <c r="DX131" s="1"/>
+      <c r="DY131" s="1"/>
+      <c r="DZ131" s="1"/>
+      <c r="EA131" s="1"/>
+      <c r="EB131" s="1"/>
+      <c r="EC131" s="1"/>
+      <c r="ED131" s="1"/>
+      <c r="EE131" s="1"/>
     </row>
-    <row r="132" spans="1:124">
+    <row r="132" spans="1:135">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
@@ -18240,8 +19780,19 @@
       <c r="DR132" s="1"/>
       <c r="DS132" s="1"/>
       <c r="DT132" s="1"/>
+      <c r="DU132" s="1"/>
+      <c r="DV132" s="1"/>
+      <c r="DW132" s="1"/>
+      <c r="DX132" s="1"/>
+      <c r="DY132" s="1"/>
+      <c r="DZ132" s="1"/>
+      <c r="EA132" s="1"/>
+      <c r="EB132" s="1"/>
+      <c r="EC132" s="1"/>
+      <c r="ED132" s="1"/>
+      <c r="EE132" s="1"/>
     </row>
-    <row r="133" spans="1:124">
+    <row r="133" spans="1:135">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
@@ -18366,8 +19917,19 @@
       <c r="DR133" s="1"/>
       <c r="DS133" s="1"/>
       <c r="DT133" s="1"/>
+      <c r="DU133" s="1"/>
+      <c r="DV133" s="1"/>
+      <c r="DW133" s="1"/>
+      <c r="DX133" s="1"/>
+      <c r="DY133" s="1"/>
+      <c r="DZ133" s="1"/>
+      <c r="EA133" s="1"/>
+      <c r="EB133" s="1"/>
+      <c r="EC133" s="1"/>
+      <c r="ED133" s="1"/>
+      <c r="EE133" s="1"/>
     </row>
-    <row r="134" spans="1:124">
+    <row r="134" spans="1:135">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
@@ -18492,8 +20054,19 @@
       <c r="DR134" s="1"/>
       <c r="DS134" s="1"/>
       <c r="DT134" s="1"/>
+      <c r="DU134" s="1"/>
+      <c r="DV134" s="1"/>
+      <c r="DW134" s="1"/>
+      <c r="DX134" s="1"/>
+      <c r="DY134" s="1"/>
+      <c r="DZ134" s="1"/>
+      <c r="EA134" s="1"/>
+      <c r="EB134" s="1"/>
+      <c r="EC134" s="1"/>
+      <c r="ED134" s="1"/>
+      <c r="EE134" s="1"/>
     </row>
-    <row r="135" spans="1:124">
+    <row r="135" spans="1:135">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
@@ -18618,8 +20191,19 @@
       <c r="DR135" s="1"/>
       <c r="DS135" s="1"/>
       <c r="DT135" s="1"/>
+      <c r="DU135" s="1"/>
+      <c r="DV135" s="1"/>
+      <c r="DW135" s="1"/>
+      <c r="DX135" s="1"/>
+      <c r="DY135" s="1"/>
+      <c r="DZ135" s="1"/>
+      <c r="EA135" s="1"/>
+      <c r="EB135" s="1"/>
+      <c r="EC135" s="1"/>
+      <c r="ED135" s="1"/>
+      <c r="EE135" s="1"/>
     </row>
-    <row r="136" spans="1:124">
+    <row r="136" spans="1:135">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -18744,8 +20328,19 @@
       <c r="DR136" s="1"/>
       <c r="DS136" s="1"/>
       <c r="DT136" s="1"/>
+      <c r="DU136" s="1"/>
+      <c r="DV136" s="1"/>
+      <c r="DW136" s="1"/>
+      <c r="DX136" s="1"/>
+      <c r="DY136" s="1"/>
+      <c r="DZ136" s="1"/>
+      <c r="EA136" s="1"/>
+      <c r="EB136" s="1"/>
+      <c r="EC136" s="1"/>
+      <c r="ED136" s="1"/>
+      <c r="EE136" s="1"/>
     </row>
-    <row r="137" spans="1:124">
+    <row r="137" spans="1:135">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
@@ -18870,8 +20465,19 @@
       <c r="DR137" s="1"/>
       <c r="DS137" s="1"/>
       <c r="DT137" s="1"/>
+      <c r="DU137" s="1"/>
+      <c r="DV137" s="1"/>
+      <c r="DW137" s="1"/>
+      <c r="DX137" s="1"/>
+      <c r="DY137" s="1"/>
+      <c r="DZ137" s="1"/>
+      <c r="EA137" s="1"/>
+      <c r="EB137" s="1"/>
+      <c r="EC137" s="1"/>
+      <c r="ED137" s="1"/>
+      <c r="EE137" s="1"/>
     </row>
-    <row r="138" spans="1:124">
+    <row r="138" spans="1:135">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
@@ -18996,8 +20602,19 @@
       <c r="DR138" s="1"/>
       <c r="DS138" s="1"/>
       <c r="DT138" s="1"/>
+      <c r="DU138" s="1"/>
+      <c r="DV138" s="1"/>
+      <c r="DW138" s="1"/>
+      <c r="DX138" s="1"/>
+      <c r="DY138" s="1"/>
+      <c r="DZ138" s="1"/>
+      <c r="EA138" s="1"/>
+      <c r="EB138" s="1"/>
+      <c r="EC138" s="1"/>
+      <c r="ED138" s="1"/>
+      <c r="EE138" s="1"/>
     </row>
-    <row r="139" spans="1:124">
+    <row r="139" spans="1:135">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -19122,8 +20739,19 @@
       <c r="DR139" s="1"/>
       <c r="DS139" s="1"/>
       <c r="DT139" s="1"/>
+      <c r="DU139" s="1"/>
+      <c r="DV139" s="1"/>
+      <c r="DW139" s="1"/>
+      <c r="DX139" s="1"/>
+      <c r="DY139" s="1"/>
+      <c r="DZ139" s="1"/>
+      <c r="EA139" s="1"/>
+      <c r="EB139" s="1"/>
+      <c r="EC139" s="1"/>
+      <c r="ED139" s="1"/>
+      <c r="EE139" s="1"/>
     </row>
-    <row r="140" spans="1:124">
+    <row r="140" spans="1:135">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -19248,8 +20876,19 @@
       <c r="DR140" s="1"/>
       <c r="DS140" s="1"/>
       <c r="DT140" s="1"/>
+      <c r="DU140" s="1"/>
+      <c r="DV140" s="1"/>
+      <c r="DW140" s="1"/>
+      <c r="DX140" s="1"/>
+      <c r="DY140" s="1"/>
+      <c r="DZ140" s="1"/>
+      <c r="EA140" s="1"/>
+      <c r="EB140" s="1"/>
+      <c r="EC140" s="1"/>
+      <c r="ED140" s="1"/>
+      <c r="EE140" s="1"/>
     </row>
-    <row r="141" spans="1:124">
+    <row r="141" spans="1:135">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
@@ -19374,8 +21013,19 @@
       <c r="DR141" s="1"/>
       <c r="DS141" s="1"/>
       <c r="DT141" s="1"/>
+      <c r="DU141" s="1"/>
+      <c r="DV141" s="1"/>
+      <c r="DW141" s="1"/>
+      <c r="DX141" s="1"/>
+      <c r="DY141" s="1"/>
+      <c r="DZ141" s="1"/>
+      <c r="EA141" s="1"/>
+      <c r="EB141" s="1"/>
+      <c r="EC141" s="1"/>
+      <c r="ED141" s="1"/>
+      <c r="EE141" s="1"/>
     </row>
-    <row r="142" spans="1:124">
+    <row r="142" spans="1:135">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -19500,8 +21150,19 @@
       <c r="DR142" s="1"/>
       <c r="DS142" s="1"/>
       <c r="DT142" s="1"/>
+      <c r="DU142" s="1"/>
+      <c r="DV142" s="1"/>
+      <c r="DW142" s="1"/>
+      <c r="DX142" s="1"/>
+      <c r="DY142" s="1"/>
+      <c r="DZ142" s="1"/>
+      <c r="EA142" s="1"/>
+      <c r="EB142" s="1"/>
+      <c r="EC142" s="1"/>
+      <c r="ED142" s="1"/>
+      <c r="EE142" s="1"/>
     </row>
-    <row r="143" spans="1:124">
+    <row r="143" spans="1:135">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
@@ -19626,8 +21287,19 @@
       <c r="DR143" s="1"/>
       <c r="DS143" s="1"/>
       <c r="DT143" s="1"/>
+      <c r="DU143" s="1"/>
+      <c r="DV143" s="1"/>
+      <c r="DW143" s="1"/>
+      <c r="DX143" s="1"/>
+      <c r="DY143" s="1"/>
+      <c r="DZ143" s="1"/>
+      <c r="EA143" s="1"/>
+      <c r="EB143" s="1"/>
+      <c r="EC143" s="1"/>
+      <c r="ED143" s="1"/>
+      <c r="EE143" s="1"/>
     </row>
-    <row r="144" spans="1:124">
+    <row r="144" spans="1:135">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
@@ -19752,8 +21424,19 @@
       <c r="DR144" s="1"/>
       <c r="DS144" s="1"/>
       <c r="DT144" s="1"/>
+      <c r="DU144" s="1"/>
+      <c r="DV144" s="1"/>
+      <c r="DW144" s="1"/>
+      <c r="DX144" s="1"/>
+      <c r="DY144" s="1"/>
+      <c r="DZ144" s="1"/>
+      <c r="EA144" s="1"/>
+      <c r="EB144" s="1"/>
+      <c r="EC144" s="1"/>
+      <c r="ED144" s="1"/>
+      <c r="EE144" s="1"/>
     </row>
-    <row r="145" spans="1:124">
+    <row r="145" spans="1:135">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
@@ -19878,8 +21561,19 @@
       <c r="DR145" s="1"/>
       <c r="DS145" s="1"/>
       <c r="DT145" s="1"/>
+      <c r="DU145" s="1"/>
+      <c r="DV145" s="1"/>
+      <c r="DW145" s="1"/>
+      <c r="DX145" s="1"/>
+      <c r="DY145" s="1"/>
+      <c r="DZ145" s="1"/>
+      <c r="EA145" s="1"/>
+      <c r="EB145" s="1"/>
+      <c r="EC145" s="1"/>
+      <c r="ED145" s="1"/>
+      <c r="EE145" s="1"/>
     </row>
-    <row r="146" spans="1:124">
+    <row r="146" spans="1:135">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
@@ -20004,8 +21698,19 @@
       <c r="DR146" s="1"/>
       <c r="DS146" s="1"/>
       <c r="DT146" s="1"/>
+      <c r="DU146" s="1"/>
+      <c r="DV146" s="1"/>
+      <c r="DW146" s="1"/>
+      <c r="DX146" s="1"/>
+      <c r="DY146" s="1"/>
+      <c r="DZ146" s="1"/>
+      <c r="EA146" s="1"/>
+      <c r="EB146" s="1"/>
+      <c r="EC146" s="1"/>
+      <c r="ED146" s="1"/>
+      <c r="EE146" s="1"/>
     </row>
-    <row r="147" spans="1:124">
+    <row r="147" spans="1:135">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
@@ -20130,8 +21835,19 @@
       <c r="DR147" s="1"/>
       <c r="DS147" s="1"/>
       <c r="DT147" s="1"/>
+      <c r="DU147" s="1"/>
+      <c r="DV147" s="1"/>
+      <c r="DW147" s="1"/>
+      <c r="DX147" s="1"/>
+      <c r="DY147" s="1"/>
+      <c r="DZ147" s="1"/>
+      <c r="EA147" s="1"/>
+      <c r="EB147" s="1"/>
+      <c r="EC147" s="1"/>
+      <c r="ED147" s="1"/>
+      <c r="EE147" s="1"/>
     </row>
-    <row r="148" spans="1:124">
+    <row r="148" spans="1:135">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -20256,8 +21972,19 @@
       <c r="DR148" s="1"/>
       <c r="DS148" s="1"/>
       <c r="DT148" s="1"/>
+      <c r="DU148" s="1"/>
+      <c r="DV148" s="1"/>
+      <c r="DW148" s="1"/>
+      <c r="DX148" s="1"/>
+      <c r="DY148" s="1"/>
+      <c r="DZ148" s="1"/>
+      <c r="EA148" s="1"/>
+      <c r="EB148" s="1"/>
+      <c r="EC148" s="1"/>
+      <c r="ED148" s="1"/>
+      <c r="EE148" s="1"/>
     </row>
-    <row r="149" spans="1:124">
+    <row r="149" spans="1:135">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
@@ -20382,8 +22109,19 @@
       <c r="DR149" s="1"/>
       <c r="DS149" s="1"/>
       <c r="DT149" s="1"/>
+      <c r="DU149" s="1"/>
+      <c r="DV149" s="1"/>
+      <c r="DW149" s="1"/>
+      <c r="DX149" s="1"/>
+      <c r="DY149" s="1"/>
+      <c r="DZ149" s="1"/>
+      <c r="EA149" s="1"/>
+      <c r="EB149" s="1"/>
+      <c r="EC149" s="1"/>
+      <c r="ED149" s="1"/>
+      <c r="EE149" s="1"/>
     </row>
-    <row r="150" spans="1:124">
+    <row r="150" spans="1:135">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -20508,6 +22246,17 @@
       <c r="DR150" s="1"/>
       <c r="DS150" s="1"/>
       <c r="DT150" s="1"/>
+      <c r="DU150" s="1"/>
+      <c r="DV150" s="1"/>
+      <c r="DW150" s="1"/>
+      <c r="DX150" s="1"/>
+      <c r="DY150" s="1"/>
+      <c r="DZ150" s="1"/>
+      <c r="EA150" s="1"/>
+      <c r="EB150" s="1"/>
+      <c r="EC150" s="1"/>
+      <c r="ED150" s="1"/>
+      <c r="EE150" s="1"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>